<commit_message>
Record GitHub sync checkpoint
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -2,31 +2,31 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7b41e8cfc9b94f06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R4e91f4f2ad8e457a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="3" r:id="R799668bbbba84b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="4" r:id="Rc51cf26d47e94f0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Steps" sheetId="5" r:id="Rc0301d7362154524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardware BOM" sheetId="6" r:id="Rb39ee45984d14889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Tracker" sheetId="7" r:id="R3287170790e34443"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packet Protocol" sheetId="8" r:id="R617e485364bb4ea7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend APIs" sheetId="9" r:id="R14f36d6d7d284ff6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database Schema" sheetId="10" r:id="Rcde6d8d5e3994da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard UX" sheetId="11" r:id="R490d7470fdd54788"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI &amp; Detection" sheetId="12" r:id="R69f2494e28f248a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camera &amp; Recording" sheetId="13" r:id="Re01d49bbf4d24dcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment DevOps" sheetId="14" r:id="R59f2419573b44bc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Campaign" sheetId="15" r:id="R42d0b42303264c39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Tracker" sheetId="16" r:id="R709f149101974f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="17" r:id="R3783ad16252843c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="18" r:id="R8cc28673b038420b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="19" r:id="R0d08c7d6915447c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Diagram" sheetId="20" r:id="R7400ced3f68d41ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Flow" sheetId="21" r:id="R2cc39c1e703f4c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex GitHub Workflow" sheetId="22" r:id="R8600b9e0c23a45cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Task Prompts" sheetId="23" r:id="Re9214ce47497456f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Structure" sheetId="24" r:id="R93c43a0bdbe44d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="25" r:id="R539682468fd1482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rff29e12144624072"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R47b7e34b12e34156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="3" r:id="R0efffa2eb9924e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="4" r:id="R0536a4039ea7468c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Steps" sheetId="5" r:id="R38dc2fba812f4ccf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardware BOM" sheetId="6" r:id="R7cd3ea740b55420b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Tracker" sheetId="7" r:id="R1f112570dbc14184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packet Protocol" sheetId="8" r:id="Rbc658cb8582b4c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend APIs" sheetId="9" r:id="Rb6f40f7750d14aff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database Schema" sheetId="10" r:id="R9c0a211094494181"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard UX" sheetId="11" r:id="R5265267259bd44fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI &amp; Detection" sheetId="12" r:id="R0eb06373f9fe41ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camera &amp; Recording" sheetId="13" r:id="R02ae6d1a88874229"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment DevOps" sheetId="14" r:id="R7157da448e22414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Campaign" sheetId="15" r:id="R89d9a59c0e724548"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Tracker" sheetId="16" r:id="R99d4a9bfbebe4d1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="17" r:id="R0d27d3af62544351"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="18" r:id="R45826979007a43f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="19" r:id="R59cdad319735489a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Diagram" sheetId="20" r:id="R8b57b81a04794a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Flow" sheetId="21" r:id="Rd24689e6069c47a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex GitHub Workflow" sheetId="22" r:id="Re8e583d592bb4227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Task Prompts" sheetId="23" r:id="R31c12182ec734878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Structure" sheetId="24" r:id="Rbe8a746420dd4fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="25" r:id="R152c212398b74cfc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -348,7 +348,7 @@
       </x:c>
       <x:c r="B4" s="7" t="n">
         <x:f>COUNTIF('Progress Tracker'!D4:D200,"Done")</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -366,7 +366,7 @@
       </x:c>
       <x:c r="B6" s="7" t="n">
         <x:f>COUNTIF('Progress Tracker'!D4:D200,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -384,7 +384,7 @@
       </x:c>
       <x:c r="B8" s="7" t="str">
         <x:f>TEXT(IF(B3=0,0,B4/B3),"0%")</x:f>
-        <x:v>89%</x:v>
+        <x:v>93%</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -401,8 +401,8 @@
         <x:v>Next Action</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:f>"Provide GitHub remote URL/branch, install PlatformIO locally, or connect hardware for field validation"</x:f>
-        <x:v>Provide GitHub remote URL/branch, install PlatformIO locally, or connect hardware for field validation</x:v>
+        <x:f>"Install PlatformIO locally, enable GitHub workflow scope, or connect hardware for field validation"</x:f>
+        <x:v>Install PlatformIO locally, enable GitHub workflow scope, or connect hardware for field validation</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1535,13 +1535,13 @@
         <x:v>GitHub</x:v>
       </x:c>
       <x:c r="D10" s="17" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="E10" s="17" t="str">
         <x:v>GitHub Actions</x:v>
       </x:c>
       <x:c r="F10" s="17" t="str">
-        <x:v>Needs repo.</x:v>
+        <x:v>Workflow file exists locally but HTTPS token lacks workflow scope; pushed baseline without workflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2534,7 +2534,7 @@
         <x:v>Unit tests OK; smoke test OK; compileall OK; release zip created; git clean</x:v>
       </x:c>
       <x:c r="H27" s="17" t="str">
-        <x:v>Provide GitHub remote URL/branch, install PlatformIO locally, or connect hardware for field validation</x:v>
+        <x:v>Push to GitHub</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2545,20 +2545,22 @@
         <x:v>GitHub</x:v>
       </x:c>
       <x:c r="C28" s="17" t="str">
-        <x:v>Create/provide GitHub repo and branch</x:v>
+        <x:v>Create/provide GitHub repo and branch and push project snapshot</x:v>
       </x:c>
       <x:c r="D28" s="17" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E28" s="17" t="str">
-        <x:v>User</x:v>
-      </x:c>
-      <x:c r="F28" s="17" t="str"/>
+        <x:v>User/Codex</x:v>
+      </x:c>
+      <x:c r="F28" s="17" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
       <x:c r="G28" s="17" t="str">
-        <x:v>No remote configured</x:v>
+        <x:v>https://github.com/pagibetech/adm-firenode-forest-monitoring commit 05e1a77</x:v>
       </x:c>
       <x:c r="H28" s="17" t="str">
-        <x:v>Provide repo URL/branch</x:v>
+        <x:v>Enable workflow scope later to push CI file</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2681,133 +2683,156 @@
         <x:v>GitHub Blocker</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
-        <x:v>Local Git repo exists, but no target remote/branch was provided</x:v>
+        <x:v>Local Git repo existed without target remote/branch</x:v>
       </x:c>
       <x:c r="D5" s="17" t="str">
         <x:v>Cannot push workbook/code to GitHub yet</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>User</x:v>
+        <x:v>User/Codex</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
-        <x:v>Provide GitHub repo URL and desired branch.</x:v>
+        <x:v>GitHub repo created and baseline pushed to main at commit 05e1a77.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="17" t="str">
-        <x:v>I002</x:v>
+        <x:v>I007</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
-        <x:v>Architecture Conflict</x:v>
+        <x:v>GitHub Workflow Scope</x:v>
       </x:c>
       <x:c r="C6" s="17" t="str">
-        <x:v>Older diagram/meeting slide listed 4 thermal cameras, but latest instruction says only one thermal camera on main</x:v>
+        <x:v>HTTPS credential can push code but cannot create/update .github/workflows/ci.yml without workflow scope</x:v>
       </x:c>
       <x:c r="D6" s="17" t="str">
-        <x:v>Could cause BOM/design mismatch</x:v>
+        <x:v>CI workflow is preserved locally but not yet on GitHub</x:v>
       </x:c>
       <x:c r="E6" s="17" t="str">
-        <x:v>Codex</x:v>
+        <x:v>User/Codex</x:v>
       </x:c>
       <x:c r="F6" s="17" t="str">
-        <x:v>Resolved</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="G6" s="17" t="str">
-        <x:v>Workbook uses latest instruction as controlling requirement.</x:v>
+        <x:v>Enable workflow scope or install GitHub app permissions, then push .github/workflows/ci.yml.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="17" t="str">
-        <x:v>I003</x:v>
+        <x:v>I002</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>Protocol Gap</x:v>
+        <x:v>Architecture Conflict</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
-        <x:v>Current RPi ZIPs poll ESP32 over Wi-Fi and do not implement real LoRa gateway receive path</x:v>
+        <x:v>Older diagram/meeting slide listed 4 thermal cameras, but latest instruction says only one thermal camera on main</x:v>
       </x:c>
       <x:c r="D7" s="17" t="str">
-        <x:v>LoRa validation cannot pass yet</x:v>
+        <x:v>Could cause BOM/design mismatch</x:v>
       </x:c>
       <x:c r="E7" s="17" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="G7" s="17" t="str">
-        <x:v>Add LoRa receiver and packet store.</x:v>
+        <x:v>Workbook uses latest instruction as controlling requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="17" t="str">
-        <x:v>I004</x:v>
+        <x:v>I003</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>Power Detail</x:v>
+        <x:v>Protocol Gap</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
-        <x:v>12V 40A was specified, but battery chemistry/capacity in Ah not confirmed</x:v>
+        <x:v>Current RPi ZIPs poll ESP32 over Wi-Fi and do not implement real LoRa gateway receive path</x:v>
       </x:c>
       <x:c r="D8" s="17" t="str">
-        <x:v>Runtime and low-voltage thresholds uncertain</x:v>
+        <x:v>LoRa validation cannot pass yet</x:v>
       </x:c>
       <x:c r="E8" s="17" t="str">
-        <x:v>User</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="F8" s="17" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G8" s="17" t="str">
-        <x:v>Confirm battery chemistry and Ah rating.</x:v>
+        <x:v>Add LoRa receiver and packet store.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="17" t="str">
-        <x:v>I005</x:v>
+        <x:v>I004</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>Field Audio</x:v>
+        <x:v>Power Detail</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
-        <x:v>No real chainsaw/forest dataset confirmed</x:v>
+        <x:v>12V 40A was specified, but battery chemistry/capacity in Ah not confirmed</x:v>
       </x:c>
       <x:c r="D9" s="17" t="str">
-        <x:v>ML classifier cannot be validated yet</x:v>
+        <x:v>Runtime and low-voltage thresholds uncertain</x:v>
       </x:c>
       <x:c r="E9" s="17" t="str">
-        <x:v>User/Codex</x:v>
+        <x:v>User</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">
-        <x:v>Start with existing detector and collect field clips.</x:v>
+        <x:v>Confirm battery chemistry and Ah rating.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="17" t="str">
+        <x:v>I005</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>Field Audio</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>No real chainsaw/forest dataset confirmed</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>ML classifier cannot be validated yet</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="str">
+        <x:v>User/Codex</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="G10" s="17" t="str">
+        <x:v>Start with existing detector and collect field clips.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="17" t="str">
         <x:v>I006</x:v>
       </x:c>
-      <x:c r="B10" s="17" t="str">
+      <x:c r="B11" s="17" t="str">
         <x:v>Simulation Gap</x:v>
       </x:c>
-      <x:c r="C10" s="17" t="str">
+      <x:c r="C11" s="17" t="str">
         <x:v>Local main camera reported cv2 missing in the macOS venv while remote node camera simulation worked</x:v>
       </x:c>
-      <x:c r="D10" s="17" t="str">
+      <x:c r="D11" s="17" t="str">
         <x:v>Camera-grid test was not complete until local fallback feed worked without hardware</x:v>
       </x:c>
-      <x:c r="E10" s="17" t="str">
+      <x:c r="E11" s="17" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="F10" s="17" t="str">
+      <x:c r="F11" s="17" t="str">
         <x:v>Resolved</x:v>
       </x:c>
-      <x:c r="G10" s="17" t="str">
+      <x:c r="G11" s="17" t="str">
         <x:v>Added PIL-based local camera fallback for simulation mode; live mode still uses OpenCV on Raspberry Pi.</x:v>
       </x:c>
     </x:row>
@@ -3239,13 +3264,13 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="E12" s="17" t="str">
-        <x:v>Provide repo/branch; local Git commit is available meanwhile</x:v>
+        <x:v>Repo created and project baseline pushed</x:v>
       </x:c>
       <x:c r="F12" s="17" t="str">
-        <x:v>User</x:v>
+        <x:v>User/Codex</x:v>
       </x:c>
       <x:c r="G12" s="17" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4034,10 +4059,10 @@
         <x:v>Update README and Dashboard</x:v>
       </x:c>
       <x:c r="E6" s="17" t="str">
-        <x:v>Required before push</x:v>
+        <x:v>Repo created: pagibetech/adm-firenode-forest-monitoring</x:v>
       </x:c>
       <x:c r="F6" s="17" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4114,10 +4139,10 @@
         <x:v>Record commit/PR link</x:v>
       </x:c>
       <x:c r="E10" s="17" t="str">
-        <x:v>Reviewable history</x:v>
+        <x:v>Baseline pushed to main commit 05e1a77</x:v>
       </x:c>
       <x:c r="F10" s="17" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5037,6 +5062,32 @@
         <x:v>Push to GitHub after remote is provided</x:v>
       </x:c>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="17" t="str">
+        <x:v>C021</x:v>
+      </x:c>
+      <x:c r="B25" s="17" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="C25" s="17" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="D25" s="17" t="str">
+        <x:v>Pushed project code, firmware, docs, and workbook to GitHub main; excluded CI workflow because token lacks workflow scope</x:v>
+      </x:c>
+      <x:c r="E25" s="17" t="str">
+        <x:v>Progress Tracker; Issue Log; GitHub Workflow; Change Log; workbook</x:v>
+      </x:c>
+      <x:c r="F25" s="17" t="str">
+        <x:v>git push to https://github.com/pagibetech/adm-firenode-forest-monitoring.git succeeded at commit 05e1a77</x:v>
+      </x:c>
+      <x:c r="G25" s="17" t="str">
+        <x:v>05e1a77 on GitHub</x:v>
+      </x:c>
+      <x:c r="H25" s="17" t="str">
+        <x:v>Enable workflow scope to push CI workflow later</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5328,16 +5379,16 @@
         <x:v>Local repo, workbook, raspi baseline, ESP32 baseline, simulation docs</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
         <x:v>Codex/User</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
-        <x:v>Need target GitHub repository for push</x:v>
+        <x:v>GitHub repository available</x:v>
       </x:c>
       <x:c r="H5" s="17" t="str">
-        <x:v>Local repo initialized; GitHub remote still needed.</x:v>
+        <x:v>Project snapshot pushed to GitHub; CI workflow retained locally until workflow scope is available.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -5604,10 +5655,10 @@
         <x:v>Provide or create GitHub repository and branch</x:v>
       </x:c>
       <x:c r="D6" s="17" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E6" s="17" t="str">
-        <x:v>User</x:v>
+        <x:v>User/Codex</x:v>
       </x:c>
       <x:c r="F6" s="17" t="str">
         <x:v>None</x:v>
@@ -5616,7 +5667,7 @@
         <x:v>Repo URL and branch</x:v>
       </x:c>
       <x:c r="H6" s="17" t="str">
-        <x:v>Local Git repo exists; remote still needed</x:v>
+        <x:v>Pushed baseline to GitHub main</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>

<commit_message>
Add low-cost AI workflow sheets
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -2,31 +2,46 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rff29e12144624072"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R47b7e34b12e34156"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="3" r:id="R0efffa2eb9924e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="4" r:id="R0536a4039ea7468c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Steps" sheetId="5" r:id="R38dc2fba812f4ccf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardware BOM" sheetId="6" r:id="R7cd3ea740b55420b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Tracker" sheetId="7" r:id="R1f112570dbc14184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packet Protocol" sheetId="8" r:id="Rbc658cb8582b4c02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend APIs" sheetId="9" r:id="Rb6f40f7750d14aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database Schema" sheetId="10" r:id="R9c0a211094494181"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard UX" sheetId="11" r:id="R5265267259bd44fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI &amp; Detection" sheetId="12" r:id="R0eb06373f9fe41ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camera &amp; Recording" sheetId="13" r:id="R02ae6d1a88874229"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment DevOps" sheetId="14" r:id="R7157da448e22414f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Campaign" sheetId="15" r:id="R89d9a59c0e724548"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Tracker" sheetId="16" r:id="R99d4a9bfbebe4d1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="17" r:id="R0d27d3af62544351"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="18" r:id="R45826979007a43f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="19" r:id="R59cdad319735489a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Diagram" sheetId="20" r:id="R8b57b81a04794a1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Flow" sheetId="21" r:id="Rd24689e6069c47a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex GitHub Workflow" sheetId="22" r:id="Re8e583d592bb4227"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Task Prompts" sheetId="23" r:id="R31c12182ec734878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Structure" sheetId="24" r:id="Rbe8a746420dd4fd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="25" r:id="R152c212398b74cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R503a237a369f482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R8982991f703a4370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="3" r:id="R53d8684aa4804319"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="4" r:id="R51910c8d8b744adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Steps" sheetId="5" r:id="R9d3157a77a0e42aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardware BOM" sheetId="6" r:id="R0ed9f59403f44ba6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Tracker" sheetId="7" r:id="Rc44f8632f7994595"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packet Protocol" sheetId="8" r:id="Ra09d843cc41146aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend APIs" sheetId="9" r:id="R4a76e303f1d3404a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database Schema" sheetId="10" r:id="R6faa005dc24c47b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard UX" sheetId="11" r:id="Rd892c48001e14f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI &amp; Detection" sheetId="12" r:id="Rb158e891ae374209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camera &amp; Recording" sheetId="13" r:id="R77f358369c6245ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment DevOps" sheetId="14" r:id="R06eccddd79b74755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Campaign" sheetId="15" r:id="R3589e67509c64c3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Tracker" sheetId="16" r:id="R99695de691fe4763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="17" r:id="R65d93e2c8c164a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="18" r:id="R14d6596f70b94269"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="19" r:id="R399a862089454879"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Diagram" sheetId="20" r:id="R6defdf7ca7ac46da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Flow" sheetId="21" r:id="R45b4f134f11742c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex GitHub Workflow" sheetId="22" r:id="Rc800bf2b6217483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Task Prompts" sheetId="23" r:id="Rcb1cf936ce994746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Context Snapshot" sheetId="24" r:id="Re954e759bbe04c1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Session Handoff" sheetId="25" r:id="Ra7d4536f10a34b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Library" sheetId="26" r:id="Rdb800e391f4b4185"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Validation Matrix" sheetId="27" r:id="R866f9bc958f04fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment Snapshot" sheetId="28" r:id="R2ca33ee69e644e1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Stack" sheetId="29" r:id="Ra590b167dc6b4e9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Router" sheetId="30" r:id="R392d0ec0706740ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Model Routing Log" sheetId="31" r:id="R2d47a754735146c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Task Log" sheetId="32" r:id="R62844952db1c45cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Software Dependencies" sheetId="33" r:id="R03cd6f9b49474f49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulation Plan" sheetId="34" r:id="R4701dfa2da1248cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Procedures" sheetId="35" r:id="R74863192eda7488a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Issues" sheetId="36" r:id="Rca8cf42776734ca5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Troubleshooting Logs" sheetId="37" r:id="Rcc19704596074d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuation Instructions" sheetId="38" r:id="R676979c35358467a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Structure" sheetId="39" r:id="R19d8d0df10704cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="40" r:id="R9427c0b5127e4ae7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -339,7 +354,7 @@
       </x:c>
       <x:c r="B3" s="7" t="n">
         <x:f>COUNTA('Progress Tracker'!A4:A200)</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -348,7 +363,7 @@
       </x:c>
       <x:c r="B4" s="7" t="n">
         <x:f>COUNTIF('Progress Tracker'!D4:D200,"Done")</x:f>
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -392,8 +407,8 @@
         <x:v>Current Stage</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:f>"Simulation baseline verified"</x:f>
-        <x:v>Simulation baseline verified</x:v>
+        <x:f>"GitHub baseline synced; low-cost AI workflow added"</x:f>
+        <x:v>GitHub baseline synced; low-cost AI workflow added</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -401,8 +416,8 @@
         <x:v>Next Action</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:f>"Install PlatformIO locally, enable GitHub workflow scope, or connect hardware for field validation"</x:f>
-        <x:v>Install PlatformIO locally, enable GitHub workflow scope, or connect hardware for field validation</x:v>
+        <x:f>"Use local machine/PlatformIO for firmware validation, then hardware field validation"</x:f>
+        <x:v>Use local machine/PlatformIO for firmware validation, then hardware field validation</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -460,7 +475,7 @@
         <x:v>Codex/User</x:v>
       </x:c>
       <x:c r="F14" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G14" s="17" t="str">
         <x:v>User clarification 2026-05-13; Zoom transcript; FireDiagram.png</x:v>
@@ -486,7 +501,7 @@
         <x:v>Codex/User</x:v>
       </x:c>
       <x:c r="F15" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G15" s="17" t="str">
         <x:v>Details-protoLORA.pdf; Zoom transcript</x:v>
@@ -512,7 +527,7 @@
         <x:v>Codex/User</x:v>
       </x:c>
       <x:c r="F16" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G16" s="17" t="str">
         <x:v>Zoom transcript and user clarification</x:v>
@@ -538,7 +553,7 @@
         <x:v>User</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
         <x:v>User clarification</x:v>
@@ -564,7 +579,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F18" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G18" s="17" t="str">
         <x:v>firenode RPi ZIPs</x:v>
@@ -590,7 +605,7 @@
         <x:v>User</x:v>
       </x:c>
       <x:c r="F19" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G19" s="17" t="str">
         <x:v>User clarification</x:v>
@@ -1930,7 +1945,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F4" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G4" s="17" t="str">
         <x:v>Chat analysis and artifacts</x:v>
@@ -1956,7 +1971,7 @@
         <x:v>Codex/User</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
         <x:v>User clarification answers</x:v>
@@ -1982,7 +1997,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F6" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G6" s="17" t="str">
         <x:v>ADM_FireNode_Implementation_Workbook.xlsx</x:v>
@@ -2008,7 +2023,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G7" s="17" t="str">
         <x:v>git init; .gitignore</x:v>
@@ -2034,7 +2049,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F8" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G8" s="17" t="str">
         <x:v>raspi/firenode-system; firmware/esp32-firenode</x:v>
@@ -2060,7 +2075,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">
         <x:v>simulation/README.md; scripts/start_main_simulation.sh</x:v>
@@ -2086,7 +2101,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F10" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G10" s="17" t="str">
         <x:v>HTTP 200 on /; /api/server-dashboard shows 4 nodes and 3 simulated remotes</x:v>
@@ -2112,7 +2127,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F11" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G11" s="17" t="str">
         <x:v>/api/server-dashboard local camera running=true simulation=true; /video_feed/0 returns MJPEG</x:v>
@@ -2138,7 +2153,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F12" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G12" s="17" t="str">
         <x:v>/api/lora/status shows 4 active nodes and packet history; dashboard node JSON includes lora object</x:v>
@@ -2164,7 +2179,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F13" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G13" s="17" t="str">
         <x:v>/api/lora/packets returns stored packet rows; /api/lora/ingest accepts future gateway packets</x:v>
@@ -2190,7 +2205,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F14" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G14" s="17" t="str">
         <x:v>lora_gateway_serial.py compiles; pyserial added to requirements</x:v>
@@ -2216,7 +2231,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F15" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G15" s="17" t="str">
         <x:v>firmware/esp32-lora-gateway; parser smoke test ignores gateway status and accepts packets</x:v>
@@ -2242,7 +2257,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F16" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G16" s="17" t="str">
         <x:v>./scripts/run_raspi_tests.sh ran 4 tests OK</x:v>
@@ -2268,7 +2283,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
         <x:v>./scripts/run_raspi_tests.sh ran 5 tests OK; /api/recordings added</x:v>
@@ -2294,7 +2309,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F18" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G18" s="17" t="str">
         <x:v>/ returned 200; /api/recordings returned JSON; tests passed</x:v>
@@ -2320,7 +2335,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F19" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G19" s="17" t="str">
         <x:v>.github/workflows/ci.yml; local Python tests passed; PlatformIO not installed locally</x:v>
@@ -2346,7 +2361,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F20" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G20" s="17" t="str">
         <x:v>bash -n service scripts; README updated</x:v>
@@ -2372,7 +2387,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F21" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G21" s="17" t="str">
         <x:v>./scripts/smoke_test_main_simulation.py passed; added to CI</x:v>
@@ -2398,7 +2413,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F22" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G22" s="17" t="str">
         <x:v>docs/deployment/field_deployment_checklist.md</x:v>
@@ -2424,7 +2439,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F23" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G23" s="17" t="str">
         <x:v>docs/hardware/wiring_reference.md</x:v>
@@ -2450,7 +2465,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F24" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G24" s="17" t="str">
         <x:v>README.md</x:v>
@@ -2476,7 +2491,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F25" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G25" s="17" t="str">
         <x:v>./scripts/package_release.sh created dist/adm-firenode-b658810-20260514-140648.zip</x:v>
@@ -2502,7 +2517,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F26" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G26" s="17" t="str">
         <x:v>docs/api/lora_packet_schema.md; README.md</x:v>
@@ -2528,7 +2543,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F27" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G27" s="17" t="str">
         <x:v>Unit tests OK; smoke test OK; compileall OK; release zip created; git clean</x:v>
@@ -2539,71 +2554,97 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="17" t="str">
-        <x:v>P007</x:v>
+        <x:v>P028</x:v>
       </x:c>
       <x:c r="B28" s="17" t="str">
-        <x:v>GitHub</x:v>
+        <x:v>AI Workflow</x:v>
       </x:c>
       <x:c r="C28" s="17" t="str">
-        <x:v>Create/provide GitHub repo and branch and push project snapshot</x:v>
+        <x:v>Add hybrid low-cost AI workflow memory sheets to workbook</x:v>
       </x:c>
       <x:c r="D28" s="17" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="E28" s="17" t="str">
-        <x:v>User/Codex</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="F28" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G28" s="17" t="str">
-        <x:v>https://github.com/pagibetech/adm-firenode-forest-monitoring commit 05e1a77</x:v>
+        <x:v>AI Stack; AI Router; Active Context Snapshot; Handoff; Prompt Library; Validation Matrix; Logs</x:v>
       </x:c>
       <x:c r="H28" s="17" t="str">
-        <x:v>Enable workflow scope later to push CI file</x:v>
+        <x:v>Use workbook + GitHub as persistent memory</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="17" t="str">
-        <x:v>P008</x:v>
+        <x:v>P007</x:v>
       </x:c>
       <x:c r="B29" s="17" t="str">
-        <x:v>LoRa Gateway</x:v>
+        <x:v>GitHub</x:v>
       </x:c>
       <x:c r="C29" s="17" t="str">
-        <x:v>Add main RPi LoRa receiver service</x:v>
+        <x:v>Create/provide GitHub repo and branch and push project snapshot</x:v>
       </x:c>
       <x:c r="D29" s="17" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E29" s="17" t="str">
-        <x:v>Codex/User</x:v>
-      </x:c>
-      <x:c r="F29" s="17" t="str"/>
-      <x:c r="G29" s="17" t="str"/>
+        <x:v>User/Codex</x:v>
+      </x:c>
+      <x:c r="F29" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="G29" s="17" t="str">
+        <x:v>https://github.com/pagibetech/adm-firenode-forest-monitoring commit 05e1a77</x:v>
+      </x:c>
       <x:c r="H29" s="17" t="str">
-        <x:v>Use simulator packet contract as receiver API target</x:v>
+        <x:v>Enable workflow scope later to push CI file</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="17" t="str">
-        <x:v>P009</x:v>
+        <x:v>P008</x:v>
       </x:c>
       <x:c r="B30" s="17" t="str">
-        <x:v>Recording</x:v>
+        <x:v>LoRa Gateway</x:v>
       </x:c>
       <x:c r="C30" s="17" t="str">
-        <x:v>Add camera recording on chainsaw detection</x:v>
+        <x:v>Add main RPi LoRa receiver service</x:v>
       </x:c>
       <x:c r="D30" s="17" t="str">
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="E30" s="17" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex/User</x:v>
       </x:c>
       <x:c r="F30" s="17" t="str"/>
       <x:c r="G30" s="17" t="str"/>
       <x:c r="H30" s="17" t="str">
+        <x:v>Use simulator packet contract as receiver API target</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="17" t="str">
+        <x:v>P009</x:v>
+      </x:c>
+      <x:c r="B31" s="17" t="str">
+        <x:v>Recording</x:v>
+      </x:c>
+      <x:c r="C31" s="17" t="str">
+        <x:v>Add camera recording on chainsaw detection</x:v>
+      </x:c>
+      <x:c r="D31" s="17" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E31" s="17" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="F31" s="17" t="str"/>
+      <x:c r="G31" s="17" t="str"/>
+      <x:c r="H31" s="17" t="str">
         <x:v>Implement after simulation camera feeds are stable</x:v>
       </x:c>
     </x:row>
@@ -2906,7 +2947,7 @@
         <x:v>D001</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
         <x:v>Main server is physically installed on the center/backup field node</x:v>
@@ -2926,7 +2967,7 @@
         <x:v>D002</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="C6" s="17" t="str">
         <x:v>Remote nodes are Raspberry Pi + ESP32 nodes</x:v>
@@ -2946,7 +2987,7 @@
         <x:v>D003</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
         <x:v>Use existing RPi chainsaw detector as baseline and improve it</x:v>
@@ -2966,7 +3007,7 @@
         <x:v>D004</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
         <x:v>Every node and main server has a daytime camera</x:v>
@@ -2986,7 +3027,7 @@
         <x:v>D005</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
         <x:v>Every node/main server has a 12V battery system</x:v>
@@ -3006,7 +3047,7 @@
         <x:v>D006</x:v>
       </x:c>
       <x:c r="B10" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="C10" s="17" t="str">
         <x:v>LoRa for sensors, Wi-Fi for camera/dashboard</x:v>
@@ -4279,7 +4320,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Repo Structure</x:v>
+        <x:v>Active Context Snapshot</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -4291,7 +4332,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>Proposed GitHub repository layout.</x:v>
+        <x:v>Rapid recovery snapshot for model switching, broken chats, and low-cost continuation.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -4303,172 +4344,134 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="16" t="str">
-        <x:v>Path</x:v>
+        <x:v>Field</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>Purpose</x:v>
+        <x:v>Current Value</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>Initial Source</x:v>
-      </x:c>
-      <x:c r="D4" s="16" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="E4" s="16" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="17" t="str">
-        <x:v>docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx</x:v>
+        <x:v>Project</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>Living project reference</x:v>
+        <x:v>ADM FireNode Forest Monitoring System</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
-        <x:v>Created by Codex</x:v>
-      </x:c>
-      <x:c r="D5" s="17" t="str">
-        <x:v>Created Locally</x:v>
-      </x:c>
-      <x:c r="E5" s="17" t="str">
-        <x:v>Commit once repo exists.</x:v>
+        <x:v>Hybrid LoRa + Wi-Fi forest fire/logging monitoring prototype.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="17" t="str">
-        <x:v>docs/artifacts/</x:v>
+        <x:v>Repo</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
-        <x:v>PDF/PNG/meeting references or summaries</x:v>
+        <x:v>https://github.com/pagibetech/adm-firenode-forest-monitoring</x:v>
       </x:c>
       <x:c r="C6" s="17" t="str">
-        <x:v>User artifacts</x:v>
-      </x:c>
-      <x:c r="D6" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E6" s="17" t="str">
-        <x:v>Avoid committing huge video unless desired; store transcript/summary.</x:v>
+        <x:v>GitHub main currently contains baseline without CI workflow due token workflow-scope limit.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="17" t="str">
-        <x:v>firmware/esp32-firenode/</x:v>
+        <x:v>Local Repo Path</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>ESP32 sensor + LoRa firmware</x:v>
+        <x:v>/Users/macbookm1max321tb/A_Design/A_Coding/ADM Fire</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
-        <x:v>ESP/FireNode_ESP32_v5</x:v>
-      </x:c>
-      <x:c r="D7" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E7" s="17" t="str">
-        <x:v>PlatformIO project.</x:v>
+        <x:v>Use workbook + repo before any implementation.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="17" t="str">
-        <x:v>raspi/firenode-system/</x:v>
+        <x:v>Workbook</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>Main/node Flask app</x:v>
+        <x:v>docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
-        <x:v>RPi v4 ZIP</x:v>
-      </x:c>
-      <x:c r="D8" s="17" t="str">
-        <x:v>Created Locally</x:v>
-      </x:c>
-      <x:c r="E8" s="17" t="str">
-        <x:v>Refactor role-specific config.</x:v>
+        <x:v>Persistent project memory.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="17" t="str">
-        <x:v>raspi/services/lora_gateway.py</x:v>
+        <x:v>Current Branch</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>Main LoRa receiver service</x:v>
+        <x:v>main</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="D9" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E9" s="17" t="str">
-        <x:v>SPI or serial bridge.</x:v>
+        <x:v>Local branch has full history; remote main has pushed project snapshot.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="17" t="str">
-        <x:v>raspi/services/recorder.py</x:v>
+        <x:v>Latest Completed Step</x:v>
       </x:c>
       <x:c r="B10" s="17" t="str">
-        <x:v>Camera event recording worker</x:v>
+        <x:v>GitHub baseline sync + hybrid low-cost AI workflow workbook update</x:v>
       </x:c>
       <x:c r="C10" s="17" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="D10" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E10" s="17" t="str">
-        <x:v>ffmpeg/OpenCV.</x:v>
+        <x:v>Workbook update requested 2026-05-15.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="17" t="str">
-        <x:v>raspi/tests/</x:v>
+        <x:v>Current Active Milestone</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>Unit/integration tests</x:v>
+        <x:v>Post-simulation validation / hardware readiness</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="D11" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E11" s="17" t="str">
-        <x:v>Mock hardware where possible.</x:v>
+        <x:v>Next work should be local PlatformIO build, workflow-scope fix, or hardware validation.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="17" t="str">
-        <x:v>.github/workflows/ci.yml</x:v>
+        <x:v>Current Active Feature</x:v>
       </x:c>
       <x:c r="B12" s="17" t="str">
-        <x:v>Python + PlatformIO CI</x:v>
+        <x:v>LoRa simulation, gateway adapter, event recording, docs complete for simulation stage</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="D12" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E12" s="17" t="str">
-        <x:v>After repo exists.</x:v>
+        <x:v>Avoid new features until toolchain/hardware validation is done.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="17" t="str">
-        <x:v>README.md</x:v>
+        <x:v>Latest Unresolved Issue</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>Project overview and run instructions</x:v>
+        <x:v>GitHub workflow file not pushed because credential lacks workflow scope</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="D13" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E13" s="17" t="str">
-        <x:v>Should link workbook.</x:v>
+        <x:v>Enable workflow scope or push CI from a properly scoped token.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="17" t="str">
+        <x:v>Testing State</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>Python unit tests and simulation smoke test passed locally</x:v>
+      </x:c>
+      <x:c r="C14" s="17" t="str">
+        <x:v>PlatformIO compile not run locally because pio is unavailable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="17" t="str">
+        <x:v>Recommended Tool Now</x:v>
+      </x:c>
+      <x:c r="B15" s="17" t="str">
+        <x:v>Local machine / PlatformIO / hardware bench</x:v>
+      </x:c>
+      <x:c r="C15" s="17" t="str">
+        <x:v>Codex only for focused repo execution fixes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4494,7 +4497,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Change Log</x:v>
+        <x:v>AI Session Handoff</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -4506,7 +4509,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>Chronological log of workbook/code changes.</x:v>
+        <x:v>Current assumptions, unfinished work, and model handoff guidance.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -4518,574 +4521,813 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="16" t="str">
-        <x:v>Change ID</x:v>
+        <x:v>Item</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>Date</x:v>
+        <x:v>Status</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>Type</x:v>
+        <x:v>Owner / Tool</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
-        <x:v>Summary</x:v>
-      </x:c>
-      <x:c r="E4" s="16" t="str">
-        <x:v>Files / Sheets</x:v>
-      </x:c>
-      <x:c r="F4" s="16" t="str">
-        <x:v>Tests / Verification</x:v>
-      </x:c>
-      <x:c r="G4" s="16" t="str">
-        <x:v>Git Commit / PR</x:v>
-      </x:c>
-      <x:c r="H4" s="16" t="str">
-        <x:v>Next Step</x:v>
+        <x:v>Expected Output</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="17" t="str">
-        <x:v>C001</x:v>
+        <x:v>Unfinished: push CI workflow</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
-        <x:v>Workbook</x:v>
+        <x:v>Local machine or Codex after workflow scope</x:v>
       </x:c>
       <x:c r="D5" s="17" t="str">
-        <x:v>Created ADM FireNode implementation workbook from reference format and all gathered FireNode requirements</x:v>
-      </x:c>
-      <x:c r="E5" s="17" t="str">
-        <x:v>All workbook sheets</x:v>
-      </x:c>
-      <x:c r="F5" s="17" t="str">
-        <x:v>Workbook inspected/rendered locally</x:v>
-      </x:c>
-      <x:c r="G5" s="17" t="str">
-        <x:v>Pending GitHub repo</x:v>
-      </x:c>
-      <x:c r="H5" s="17" t="str">
-        <x:v>Provide repo/branch and commit workbook</x:v>
+        <x:v>.github/workflows/ci.yml on GitHub.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="17" t="str">
-        <x:v>C002</x:v>
+        <x:v>Unfinished: PlatformIO firmware build</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="C6" s="17" t="str">
-        <x:v>Repository</x:v>
+        <x:v>Local machine / VS Code PlatformIO</x:v>
       </x:c>
       <x:c r="D6" s="17" t="str">
-        <x:v>Initialized local Git repo, created clean baseline folders, imported RPi v4 app and ESP32 v5 firmware, added simulation start docs/script</x:v>
-      </x:c>
-      <x:c r="E6" s="17" t="str">
-        <x:v>.gitignore; README.md; raspi/; firmware/; simulation/; scripts/; docs/artifacts</x:v>
-      </x:c>
-      <x:c r="F6" s="17" t="str">
-        <x:v>python3 -m compileall -q raspi/firenode-system</x:v>
-      </x:c>
-      <x:c r="G6" s="17" t="str">
-        <x:v>21004de</x:v>
-      </x:c>
-      <x:c r="H6" s="17" t="str">
-        <x:v>Run simulation baseline and push after remote is provided</x:v>
+        <x:v>Build logs for firmware/esp32-firenode and firmware/esp32-lora-gateway.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="17" t="str">
-        <x:v>C003</x:v>
+        <x:v>Unfinished: hardware validation</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
-        <x:v>Simulation</x:v>
+        <x:v>Local machine + hardware bench</x:v>
       </x:c>
       <x:c r="D7" s="17" t="str">
-        <x:v>Verified main dashboard starts in simulation mode with one main node and three simulated remotes; updated start script to use local venv when present</x:v>
-      </x:c>
-      <x:c r="E7" s="17" t="str">
-        <x:v>scripts/start_main_simulation.sh; raspi/firenode-system/config.json; Progress Tracker; Issue Log; Change Log</x:v>
-      </x:c>
-      <x:c r="F7" s="17" t="str">
-        <x:v>HTTP 200 /; /api/server-dashboard returned 4 nodes and 3 remotes</x:v>
-      </x:c>
-      <x:c r="G7" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H7" s="17" t="str">
-        <x:v>Implement cv2-free local camera simulation fallback</x:v>
+        <x:v>LoRa RSSI/SNR/PDR logs, camera feed screenshots, recording evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="17" t="str">
-        <x:v>C004</x:v>
+        <x:v>Active assumption</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>Only one MLX90640 thermal camera on main/center node</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
-        <x:v>Simulation</x:v>
+        <x:v>Workbook decision D001/D004</x:v>
       </x:c>
       <x:c r="D8" s="17" t="str">
-        <x:v>Added cv2-free PIL fallback for the main node camera in simulation mode and suppressed macOS hostname warning</x:v>
-      </x:c>
-      <x:c r="E8" s="17" t="str">
-        <x:v>modules/camera_stream.py; modules/network_utils.py; app.py; Progress Tracker; Issue Log; Change Log</x:v>
-      </x:c>
-      <x:c r="F8" s="17" t="str">
-        <x:v>compileall passed; /api/server-dashboard local camera running=true simulation=true; /video_feed/0 returned MJPEG</x:v>
-      </x:c>
-      <x:c r="G8" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H8" s="17" t="str">
-        <x:v>Implement LoRa packet simulation/receiver path</x:v>
+        <x:v>Remote nodes use daytime cameras only.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="17" t="str">
-        <x:v>C005</x:v>
+        <x:v>Active assumption</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>Remote nodes are Raspberry Pi + ESP32</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
-        <x:v>LoRa Simulation</x:v>
+        <x:v>Workbook architecture</x:v>
       </x:c>
       <x:c r="D9" s="17" t="str">
-        <x:v>Added simulated LoRa receiver packet contract, dashboard fields, and API endpoint for RSSI/SNR/PDR/sequence/battery telemetry</x:v>
-      </x:c>
-      <x:c r="E9" s="17" t="str">
-        <x:v>modules/lora_simulator.py; app.py; static/app.js; simulation/README.md; scripts/start_main_simulation.sh; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F9" s="17" t="str">
-        <x:v>compileall passed; /api/lora/status active_nodes=4; /api/server-dashboard includes lora packet for main node</x:v>
-      </x:c>
-      <x:c r="G9" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H9" s="17" t="str">
-        <x:v>Implement real LoRa receiver adapter and SQLite packet store</x:v>
+        <x:v>RPi handles camera/audio; ESP32 handles sensor/LoRa.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="17" t="str">
-        <x:v>C006</x:v>
+        <x:v>Pending workbook update</x:v>
       </x:c>
       <x:c r="B10" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>Only after major validation or config change</x:v>
       </x:c>
       <x:c r="C10" s="17" t="str">
-        <x:v>LoRa Storage</x:v>
+        <x:v>Selected AI/tool</x:v>
       </x:c>
       <x:c r="D10" s="17" t="str">
-        <x:v>Added SQLite LoRa packet store plus /api/lora/packets and /api/lora/ingest so simulated and future hardware packets share persistence</x:v>
-      </x:c>
-      <x:c r="E10" s="17" t="str">
-        <x:v>modules/lora_packet_store.py; app.py; simulation/README.md; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F10" s="17" t="str">
-        <x:v>compileall passed; /api/lora/status stored_packet_count=8; /api/lora/packets returned rows</x:v>
-      </x:c>
-      <x:c r="G10" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H10" s="17" t="str">
-        <x:v>Implement real LoRa receiver adapter</x:v>
+        <x:v>Concise Progress/Issue/Build Matrix update.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="17" t="str">
-        <x:v>C007</x:v>
+        <x:v>Recommended next model</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>Local machine first; Kimi for heavy implementation; Codex for repo execution/validation</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>LoRa Gateway</x:v>
+        <x:v>AI Router</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str">
-        <x:v>Added serial gateway adapter for ESP32/SX127x JSON-line LoRa packets and documented first hardware bridge command</x:v>
-      </x:c>
-      <x:c r="E11" s="17" t="str">
-        <x:v>lora_gateway_serial.py; requirements.txt; simulation/README.md; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F11" s="17" t="str">
-        <x:v>compileall passed</x:v>
-      </x:c>
-      <x:c r="G11" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H11" s="17" t="str">
-        <x:v>Build ESP32 gateway firmware packet output</x:v>
+        <x:v>Avoid premium Codex for docs/simple edits.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Prompt Library</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Reusable prompts for low-cost model routing and continuation.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Prompt Name</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Recommended Tool</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Prompt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Roo/Kimi Implementation</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Kimi K2.6 via Roo Code</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Read workbook Active Context Snapshot and AI Session Handoff. Implement the next incomplete milestone only. Inspect only affected files. Report changed files and validation steps.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>DeepSeek Medium Fix</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>DeepSeek V3 via Roo Code</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Make a targeted medium-complexity code change. Avoid repo-wide scans. Preserve architecture and report exact files changed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>Gemini Documentation</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Gemini/Gemma API</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Draft concise documentation/workbook text for the specified section. Do not modify code. Keep output structured and low-token.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>Codex Task</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Use only for repo execution/validation. Include project context, objective, scope, validation commands, workbook update rule, and required output.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>Local Qwen Emergency</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>LM Studio Qwen</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>Offline fallback only. Make a one-file/simple fix or draft note. Do not attempt full repo analysis.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
+        <x:v>Hardware Validation Report</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>Local machine / technician</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>Run the specified hardware test and return logs, screenshots, device paths, pass/fail, and measured values for workbook entry.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Build Validation Matrix</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Current component build/runtime/deployment validation state.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Build Status</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Runtime Status</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Deployment Status</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Latest Test Result</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>Validation Command</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>Remaining Issue</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Raspberry Pi Flask app</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Pass in simulation</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>Local only</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Unit tests OK; smoke test OK</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="str">
+        <x:v>./scripts/run_raspi_tests.sh; ./scripts/smoke_test_main_simulation.py</x:v>
+      </x:c>
+      <x:c r="G5" s="17" t="str">
+        <x:v>Hardware deployment pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>LoRa packet store/API</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Pass in simulation</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Local/GitHub</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>Stored packet history verified</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>/api/lora/status; /api/lora/packets</x:v>
+      </x:c>
+      <x:c r="G6" s="17" t="str">
+        <x:v>Real serial gateway hardware pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>Event recording</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Pass for snapshot metadata</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Local/GitHub</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>Recording tests OK</x:v>
+      </x:c>
+      <x:c r="F7" s="17" t="str">
+        <x:v>./scripts/run_raspi_tests.sh</x:v>
+      </x:c>
+      <x:c r="G7" s="17" t="str">
+        <x:v>Full video clip recording future enhancement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>ESP32 sensor sender firmware</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Not locally built</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Not hardware tested</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>Source imported</x:v>
+      </x:c>
+      <x:c r="F8" s="17" t="str">
+        <x:v>pio run</x:v>
+      </x:c>
+      <x:c r="G8" s="17" t="str">
+        <x:v>PlatformIO unavailable locally</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>ESP32 LoRa gateway firmware</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>Not locally built</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>Not hardware tested</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>Source added</x:v>
+      </x:c>
+      <x:c r="F9" s="17" t="str">
+        <x:v>pio run</x:v>
+      </x:c>
+      <x:c r="G9" s="17" t="str">
+        <x:v>PlatformIO unavailable locally</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
+        <x:v>GitHub CI workflow</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>Present locally</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>Not on GitHub</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="str">
+        <x:v>Push rejected due workflow scope</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="str">
+        <x:v>git push</x:v>
+      </x:c>
+      <x:c r="G10" s="17" t="str">
+        <x:v>Need token/app with workflow scope</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Environment Snapshot</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Known local/toolchain environment details.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Current Date</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Asia/Manila workflow date.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>Local Python</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Python 3.12.11</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Observed via python3 --version.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>Bundled Node</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>v24.14.0</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Codex workspace runtime.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>PlatformIO</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Not found locally</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Install locally or rely on GitHub CI after workflow scope.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>GitHub Repo</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>pagibetech/adm-firenode-forest-monitoring</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>Private repo created by user.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
+        <x:v>Remote main</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>b09c2c6</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>Remote baseline + GitHub sync workbook checkpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="17" t="str">
+        <x:v>Local full-history branch</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="str">
+        <x:v>local-full-history-with-ci</x:v>
+      </x:c>
+      <x:c r="C11" s="17" t="str">
+        <x:v>Preserves workflow file and detailed local commits.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="17" t="str">
-        <x:v>C008</x:v>
+        <x:v>Roo Profiles Needed</x:v>
       </x:c>
       <x:c r="B12" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>Kimi Main; DeepSeek Cheap; Gemini Online; Local Qwen Emergency</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
-        <x:v>Firmware</x:v>
-      </x:c>
-      <x:c r="D12" s="17" t="str">
-        <x:v>Added dedicated ESP32 LoRa gateway firmware project that receives SX1278 packets, normalizes metadata, and emits one JSON packet per serial line</x:v>
-      </x:c>
-      <x:c r="E12" s="17" t="str">
-        <x:v>firmware/esp32-lora-gateway; lora_gateway_serial.py; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F12" s="17" t="str">
-        <x:v>Python parser smoke test passed; PlatformIO not installed locally, so firmware compile not run</x:v>
-      </x:c>
-      <x:c r="G12" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H12" s="17" t="str">
-        <x:v>Add automated tests for LoRa parser/store APIs</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="17" t="str">
-        <x:v>C009</x:v>
-      </x:c>
-      <x:c r="B13" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C13" s="17" t="str">
-        <x:v>Tests</x:v>
-      </x:c>
-      <x:c r="D13" s="17" t="str">
-        <x:v>Added unittest coverage for LoRa serial parsing, SQLite packet dedupe/history, and simulator packet metrics</x:v>
-      </x:c>
-      <x:c r="E13" s="17" t="str">
-        <x:v>raspi/firenode-system/tests/test_lora_pipeline.py; scripts/run_raspi_tests.sh; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F13" s="17" t="str">
-        <x:v>./scripts/run_raspi_tests.sh: 4 tests OK</x:v>
-      </x:c>
-      <x:c r="G13" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H13" s="17" t="str">
-        <x:v>Implement camera recording on chainsaw event</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="17" t="str">
-        <x:v>C010</x:v>
-      </x:c>
-      <x:c r="B14" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C14" s="17" t="str">
-        <x:v>Recording</x:v>
-      </x:c>
-      <x:c r="D14" s="17" t="str">
-        <x:v>Added event recorder that saves chainsaw camera snapshots plus metadata and exposes /api/recordings</x:v>
-      </x:c>
-      <x:c r="E14" s="17" t="str">
-        <x:v>modules/event_recorder.py; app.py; tests/test_lora_pipeline.py; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F14" s="17" t="str">
-        <x:v>./scripts/run_raspi_tests.sh: 5 tests OK</x:v>
-      </x:c>
-      <x:c r="G14" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H14" s="17" t="str">
-        <x:v>Add dashboard recording list</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="17" t="str">
-        <x:v>C011</x:v>
-      </x:c>
-      <x:c r="B15" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C15" s="17" t="str">
-        <x:v>Dashboard</x:v>
-      </x:c>
-      <x:c r="D15" s="17" t="str">
-        <x:v>Added recent recordings panel and /media route so chainsaw snapshots can be reviewed in the web GUI</x:v>
-      </x:c>
-      <x:c r="E15" s="17" t="str">
-        <x:v>templates/dashboard.html; static/app.js; static/style.css; app.py; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F15" s="17" t="str">
-        <x:v>./scripts/run_raspi_tests.sh: 5 tests OK; / and /api/recordings returned 200</x:v>
-      </x:c>
-      <x:c r="G15" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H15" s="17" t="str">
-        <x:v>Add CI workflow</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="17" t="str">
-        <x:v>C012</x:v>
-      </x:c>
-      <x:c r="B16" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C16" s="17" t="str">
-        <x:v>CI/CD</x:v>
-      </x:c>
-      <x:c r="D16" s="17" t="str">
-        <x:v>Added GitHub Actions workflow for Python app tests, compileall, and PlatformIO builds for sender and gateway firmware</x:v>
-      </x:c>
-      <x:c r="E16" s="17" t="str">
-        <x:v>.github/workflows/ci.yml; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F16" s="17" t="str">
-        <x:v>./scripts/run_raspi_tests.sh: 5 tests OK; PlatformIO unavailable locally</x:v>
-      </x:c>
-      <x:c r="G16" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H16" s="17" t="str">
-        <x:v>Add deployment/systemd scripts</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="17" t="str">
-        <x:v>C013</x:v>
-      </x:c>
-      <x:c r="B17" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C17" s="17" t="str">
-        <x:v>Deployment</x:v>
-      </x:c>
-      <x:c r="D17" s="17" t="str">
-        <x:v>Added systemd install/stop scripts for the LoRa serial gateway bridge and documented gateway service operations</x:v>
-      </x:c>
-      <x:c r="E17" s="17" t="str">
-        <x:v>install_lora_gateway_service.sh; stop_lora_gateway_service.sh; README.md; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F17" s="17" t="str">
-        <x:v>bash -n scripts passed; ./scripts/run_raspi_tests.sh: 5 tests OK</x:v>
-      </x:c>
-      <x:c r="G17" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H17" s="17" t="str">
-        <x:v>Add API smoke-test script</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="17" t="str">
-        <x:v>C014</x:v>
-      </x:c>
-      <x:c r="B18" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C18" s="17" t="str">
-        <x:v>Testing</x:v>
-      </x:c>
-      <x:c r="D18" s="17" t="str">
-        <x:v>Added end-to-end simulation smoke test and wired it into CI</x:v>
-      </x:c>
-      <x:c r="E18" s="17" t="str">
-        <x:v>scripts/smoke_test_main_simulation.py; .github/workflows/ci.yml; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F18" s="17" t="str">
-        <x:v>./scripts/smoke_test_main_simulation.py passed</x:v>
-      </x:c>
-      <x:c r="G18" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H18" s="17" t="str">
-        <x:v>Add field deployment checklist/docs</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="17" t="str">
-        <x:v>C015</x:v>
-      </x:c>
-      <x:c r="B19" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C19" s="17" t="str">
-        <x:v>Deployment</x:v>
-      </x:c>
-      <x:c r="D19" s="17" t="str">
-        <x:v>Added field deployment checklist covering bench prep, node install, LoRa validation, camera/recording checks, alert validation, and shutdown</x:v>
-      </x:c>
-      <x:c r="E19" s="17" t="str">
-        <x:v>docs/deployment/field_deployment_checklist.md; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F19" s="17" t="str">
-        <x:v>Documentation review</x:v>
-      </x:c>
-      <x:c r="G19" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H19" s="17" t="str">
-        <x:v>Add hardware wiring reference</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="17" t="str">
-        <x:v>C016</x:v>
-      </x:c>
-      <x:c r="B20" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C20" s="17" t="str">
-        <x:v>Hardware</x:v>
-      </x:c>
-      <x:c r="D20" s="17" t="str">
-        <x:v>Added wiring reference for ESP32 sensor sender, ESP32 LoRa gateway, main/remote Raspberry Pi devices, power notes, and open hardware decisions</x:v>
-      </x:c>
-      <x:c r="E20" s="17" t="str">
-        <x:v>docs/hardware/wiring_reference.md; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F20" s="17" t="str">
-        <x:v>Documentation review</x:v>
-      </x:c>
-      <x:c r="G20" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H20" s="17" t="str">
-        <x:v>Add README links to new docs</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="17" t="str">
-        <x:v>C017</x:v>
-      </x:c>
-      <x:c r="B21" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C21" s="17" t="str">
-        <x:v>Documentation</x:v>
-      </x:c>
-      <x:c r="D21" s="17" t="str">
-        <x:v>Updated top-level README with fast start commands, current build path, and links to key project references</x:v>
-      </x:c>
-      <x:c r="E21" s="17" t="str">
-        <x:v>README.md; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F21" s="17" t="str">
-        <x:v>Documentation review</x:v>
-      </x:c>
-      <x:c r="G21" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H21" s="17" t="str">
-        <x:v>Add release/package script</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="17" t="str">
-        <x:v>C018</x:v>
-      </x:c>
-      <x:c r="B22" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C22" s="17" t="str">
-        <x:v>Release</x:v>
-      </x:c>
-      <x:c r="D22" s="17" t="str">
-        <x:v>Added release packaging script that uses git archive to create a clean zip under dist</x:v>
-      </x:c>
-      <x:c r="E22" s="17" t="str">
-        <x:v>scripts/package_release.sh; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F22" s="17" t="str">
-        <x:v>./scripts/package_release.sh produced dist zip</x:v>
-      </x:c>
-      <x:c r="G22" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H22" s="17" t="str">
-        <x:v>Add packet schema documentation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="17" t="str">
-        <x:v>C019</x:v>
-      </x:c>
-      <x:c r="B23" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C23" s="17" t="str">
-        <x:v>Documentation</x:v>
-      </x:c>
-      <x:c r="D23" s="17" t="str">
-        <x:v>Added LoRa sender payload, gateway serial line, ingest/history/status API, SQLite table, and validation target schema documentation</x:v>
-      </x:c>
-      <x:c r="E23" s="17" t="str">
-        <x:v>docs/api/lora_packet_schema.md; README.md; Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F23" s="17" t="str">
-        <x:v>Documentation review</x:v>
-      </x:c>
-      <x:c r="G23" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H23" s="17" t="str">
-        <x:v>Run full local verification</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="17" t="str">
-        <x:v>C020</x:v>
-      </x:c>
-      <x:c r="B24" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C24" s="17" t="str">
-        <x:v>Verification</x:v>
-      </x:c>
-      <x:c r="D24" s="17" t="str">
-        <x:v>Completed full local verification checkpoint after unblocked development steps</x:v>
-      </x:c>
-      <x:c r="E24" s="17" t="str">
-        <x:v>Progress Tracker; Change Log</x:v>
-      </x:c>
-      <x:c r="F24" s="17" t="str">
-        <x:v>./scripts/run_raspi_tests.sh OK; ./scripts/smoke_test_main_simulation.py OK; python3 -m compileall OK; package_release produced dist/adm-firenode-192b1c7-20260514-141016.zip</x:v>
-      </x:c>
-      <x:c r="G24" s="17" t="str">
-        <x:v>Pending commit</x:v>
-      </x:c>
-      <x:c r="H24" s="17" t="str">
-        <x:v>Push to GitHub after remote is provided</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="17" t="str">
-        <x:v>C021</x:v>
-      </x:c>
-      <x:c r="B25" s="17" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="C25" s="17" t="str">
-        <x:v>GitHub</x:v>
-      </x:c>
-      <x:c r="D25" s="17" t="str">
-        <x:v>Pushed project code, firmware, docs, and workbook to GitHub main; excluded CI workflow because token lacks workflow scope</x:v>
-      </x:c>
-      <x:c r="E25" s="17" t="str">
-        <x:v>Progress Tracker; Issue Log; GitHub Workflow; Change Log; workbook</x:v>
-      </x:c>
-      <x:c r="F25" s="17" t="str">
-        <x:v>git push to https://github.com/pagibetech/adm-firenode-forest-monitoring.git succeeded at commit 05e1a77</x:v>
-      </x:c>
-      <x:c r="G25" s="17" t="str">
-        <x:v>05e1a77 on GitHub</x:v>
-      </x:c>
-      <x:c r="H25" s="17" t="str">
-        <x:v>Enable workflow scope to push CI workflow later</x:v>
+        <x:v>Configure in VS Code/Roo Code.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>AI Stack</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Model/tool roles, routing, cost category, and limitations.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Tool / Model</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Provider / Source</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Cost Category</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Use When</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>Do Not Use For</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>Roo Profile / Fallback</x:v>
+      </x:c>
+      <x:c r="H4" s="16" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>ChatGPT</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>OpenAI ChatGPT</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Project director, planning, architecture, debugging strategy</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>Moderate</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Milestone planning, prompts, troubleshooting</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="str">
+        <x:v>Repeated repo execution/build loops</x:v>
+      </x:c>
+      <x:c r="G5" s="17" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="H5" s="17" t="str">
+        <x:v>Directs work and prepares Codex/Roo tasks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>Kimi K2.6</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Roo Code cloud model</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Primary heavy implementation and long-context coding</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Paid but lower-cost than premium execution</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>Architecture-aware multi-file implementation</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>Local runtime validation</x:v>
+      </x:c>
+      <x:c r="G6" s="17" t="str">
+        <x:v>Kimi Main</x:v>
+      </x:c>
+      <x:c r="H6" s="17" t="str">
+        <x:v>Use before Codex when direct execution is not required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>DeepSeek V3</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Roo Code cloud model</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Cheap coding backup and medium implementation</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>Medium edits, utility code, doc refinement</x:v>
+      </x:c>
+      <x:c r="F7" s="17" t="str">
+        <x:v>High-risk repo-wide changes</x:v>
+      </x:c>
+      <x:c r="G7" s="17" t="str">
+        <x:v>DeepSeek Cheap</x:v>
+      </x:c>
+      <x:c r="H7" s="17" t="str">
+        <x:v>Escalate to Kimi if context/complexity exceeds capability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>Gemini / Gemma API</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Google AI Studio/API</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Low-cost docs, summaries, simple notes, prompt cleanup</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>Free/low</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>Documentation and lightweight planning</x:v>
+      </x:c>
+      <x:c r="F8" s="17" t="str">
+        <x:v>Complex repo-aware implementation</x:v>
+      </x:c>
+      <x:c r="G8" s="17" t="str">
+        <x:v>Gemini Online</x:v>
+      </x:c>
+      <x:c r="H8" s="17" t="str">
+        <x:v>Preferred for workbook text drafts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>OpenAI Codex</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>Premium repo execution, tests, validation, difficult multi-file fixes</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>Premium</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>Terminal validation, dependency-aware debugging, focused repo edits</x:v>
+      </x:c>
+      <x:c r="F9" s="17" t="str">
+        <x:v>Simple docs/snippets/workbook-only work</x:v>
+      </x:c>
+      <x:c r="G9" s="17" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="H9" s="17" t="str">
+        <x:v>Use sparingly with exact scope and validation command.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
+        <x:v>Local Qwen via LM Studio</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>Local offline model</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>Emergency offline fallback</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>Local/free</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="str">
+        <x:v>Internet/API outage, one-file/simple fixes</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="str">
+        <x:v>Autonomous repo-wide tasks</x:v>
+      </x:c>
+      <x:c r="G10" s="17" t="str">
+        <x:v>Local Qwen Emergency</x:v>
+      </x:c>
+      <x:c r="H10" s="17" t="str">
+        <x:v>Avoid heavy agent mode.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5173,7 +5415,7 @@
         <x:v>PDF validation flow + client clarification</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
         <x:v>Wi-Fi camera stream remains separate.</x:v>
@@ -5196,7 +5438,7 @@
         <x:v>User answer #1</x:v>
       </x:c>
       <x:c r="F6" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G6" s="17" t="str">
         <x:v>Center node owns MLX90640.</x:v>
@@ -5219,7 +5461,7 @@
         <x:v>User answer #2</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G7" s="17" t="str">
         <x:v>Avoid ESP32-only audio classification risk.</x:v>
@@ -5242,7 +5484,7 @@
         <x:v>User answer #4</x:v>
       </x:c>
       <x:c r="F8" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G8" s="17" t="str">
         <x:v>Use fisheye or standard camera per budget/coverage.</x:v>
@@ -5265,7 +5507,7 @@
         <x:v>User constraint</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">
         <x:v>Used primarily for night/thermal event view.</x:v>
@@ -5288,10 +5530,1566 @@
         <x:v>User answer #5</x:v>
       </x:c>
       <x:c r="F10" s="17" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G10" s="17" t="str">
         <x:v>Need buck converters and fusing.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>AI Router / Model Routing Rules</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Cheapest-capable model routing and escalation rules.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Task Type</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Recommended Model / Tool</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Reason</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Escalation Target</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Cost Level</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>Allowed Scope</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>Prohibited Use</x:v>
+      </x:c>
+      <x:c r="H4" s="16" t="str">
+        <x:v>Example Prompt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Documentation/simple explanation</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Gemini/Gemma API</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Cheap and sufficient</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>DeepSeek V3</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="str">
+        <x:v>Docs, notes, workbook text</x:v>
+      </x:c>
+      <x:c r="G5" s="17" t="str">
+        <x:v>Repo-wide code edits</x:v>
+      </x:c>
+      <x:c r="H5" s="17" t="str">
+        <x:v>Draft concise deployment notes for this section.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>Medium coding</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>DeepSeek V3</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Cheap general coding</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Kimi K2.6</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>Low/Medium</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>Small multi-file or utility edits</x:v>
+      </x:c>
+      <x:c r="G6" s="17" t="str">
+        <x:v>Hard debugging with live execution</x:v>
+      </x:c>
+      <x:c r="H6" s="17" t="str">
+        <x:v>Implement targeted parser fix in these files only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>Heavy architecture-aware coding</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Kimi K2.6</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Long context and stronger implementation</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>Medium/High</x:v>
+      </x:c>
+      <x:c r="F7" s="17" t="str">
+        <x:v>Large feature design and code generation</x:v>
+      </x:c>
+      <x:c r="G7" s="17" t="str">
+        <x:v>Running local tests/builds</x:v>
+      </x:c>
+      <x:c r="H7" s="17" t="str">
+        <x:v>Implement milestone X using workbook context.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>Repo execution/testing/validation</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Requires terminal and actual repo state</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>Local machine/manual</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>Premium</x:v>
+      </x:c>
+      <x:c r="F8" s="17" t="str">
+        <x:v>Focused commands and code fixes</x:v>
+      </x:c>
+      <x:c r="G8" s="17" t="str">
+        <x:v>Simple docs/snippets</x:v>
+      </x:c>
+      <x:c r="H8" s="17" t="str">
+        <x:v>Run specified tests, fix failures, update workbook if major.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>Builds/flashing/hardware</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>Local machine</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>Primary execution environment</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>Codex only for script fixes</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>No AI cost</x:v>
+      </x:c>
+      <x:c r="F9" s="17" t="str">
+        <x:v>PlatformIO, Arduino IDE, SSH, hardware logs</x:v>
+      </x:c>
+      <x:c r="G9" s="17" t="str">
+        <x:v>Cloud AI autonomous hardware loops</x:v>
+      </x:c>
+      <x:c r="H9" s="17" t="str">
+        <x:v>Run pio and return logs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
+        <x:v>Offline emergency</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>Local Qwen</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>No internet/API needed</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>Wait for online model</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="str">
+        <x:v>Local/free</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="str">
+        <x:v>One-file/simple fixes</x:v>
+      </x:c>
+      <x:c r="G10" s="17" t="str">
+        <x:v>Full repo analysis</x:v>
+      </x:c>
+      <x:c r="H10" s="17" t="str">
+        <x:v>Patch this syntax issue only.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>AI Model Routing Log</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Record important model/tool routing decisions.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Task</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Selected Model / Tool</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Reason Selected</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>Escalation Needed</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>Next Recommended Tool</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Update workbook with hybrid low-cost AI workflow sheets</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>User explicitly requested direct workbook update in current repo</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Workbook sheets added/updated</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G5" s="17" t="str">
+        <x:v>Gemini/Gemma or DeepSeek for future workbook-only drafts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Future PlatformIO firmware build</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Local machine</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Build/flashing belongs to local execution environment</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>Only if build fails</x:v>
+      </x:c>
+      <x:c r="G6" s="17" t="str">
+        <x:v>Codex for focused failure fix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Future hardware validation</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Local machine / hardware bench</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Requires devices, serial monitor, camera, LoRa, batteries</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F7" s="17" t="str">
+        <x:v>No AI escalation until logs exist</x:v>
+      </x:c>
+      <x:c r="G7" s="17" t="str">
+        <x:v>ChatGPT for analysis or Codex for repo fix</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Codex Task Log</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Track premium Codex usage, commands, files, validation, and commits.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Task</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Repo Path</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Files Changed</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Commands Run</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>Validation Result</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>Unresolved Issues</x:v>
+      </x:c>
+      <x:c r="H4" s="16" t="str">
+        <x:v>Workbook Update</x:v>
+      </x:c>
+      <x:c r="I4" s="16" t="str">
+        <x:v>Git Commit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Add hybrid low-cost AI workflow sheets</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>/Users/macbookm1max321tb/A_Design/A_Coding/ADM Fire</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Workbook build/verify/render</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="str">
+        <x:v>Pending final push</x:v>
+      </x:c>
+      <x:c r="G5" s="17" t="str">
+        <x:v>CI workflow scope still blocked</x:v>
+      </x:c>
+      <x:c r="H5" s="17" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I5" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>GitHub baseline sync</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>/Users/macbookm1max321tb/A_Design/A_Coding/ADM Fire</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Project snapshot and workbook</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>git push via scoped-safe temp repo</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>Remote main b09c2c6</x:v>
+      </x:c>
+      <x:c r="G6" s="17" t="str">
+        <x:v>Workflow file not pushed</x:v>
+      </x:c>
+      <x:c r="H6" s="17" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I6" s="17" t="str">
+        <x:v>b09c2c6 remote</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Software / Dependency Tracker</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Runtime and toolchain dependency state.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Dependency</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Required Version / Source</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Current Status</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Install / Validation Command</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Raspberry Pi app</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Python</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>3.x on Raspberry Pi OS</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>Local Python 3.12.11 observed</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>python3 --version</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="str">
+        <x:v>RPi target may differ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>Raspberry Pi app</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Flask, requests, Pillow, pyserial</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>requirements.txt</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Configured</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>pip install -r requirements.txt</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>OpenCV/sounddevice normally installed via setup/apt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>ESP32 firmware</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>PlatformIO</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Latest compatible</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Not installed locally</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>pio run</x:v>
+      </x:c>
+      <x:c r="F7" s="17" t="str">
+        <x:v>Install in VS Code/PlatformIO.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>ESP32 firmware</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>LoRa library</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>sandeepmistry/LoRa</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>Configured</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>pio run</x:v>
+      </x:c>
+      <x:c r="F8" s="17" t="str">
+        <x:v>Used by sender and gateway.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>Workbook</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>@oai/artifact-tool</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>Codex bundled spreadsheet runtime</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>Available in Codex</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>Workbook builder/verify</x:v>
+      </x:c>
+      <x:c r="F9" s="17" t="str">
+        <x:v>Used only for workbook generation.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Simulation Plan</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Current simulation coverage and next validation steps.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Area</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Current Simulation Coverage</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Validation Command / Endpoint</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Next Step</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Dashboard</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Main + 3 remote simulated nodes</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>./scripts/smoke_test_main_simulation.py</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Use for demos before hardware.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>Camera</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>PIL fallback local camera + remote simulated feeds</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>/video_feed/0; dashboard</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>Validate real camera hardware on RPi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>Thermal</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>MLX90640 simulation fallback</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>/thermal_feed</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>Validate real MLX90640 on main node.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>LoRa</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Simulated packets with seq/RSSI/SNR/PDR/battery</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>/api/lora/status</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>Validate ESP32 gateway serial bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>Recording</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>Snapshot metadata on chainsaw event path</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>/api/recordings</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>Validate real chainsaw trigger and camera snapshot.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Validation Procedures</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Procedures for local, CI, and hardware validation.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Where To Run</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Command / Procedure</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Evidence To Save</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>Python unit tests</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Local machine or CI</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>./scripts/run_raspi_tests.sh</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>All tests OK</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Terminal output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>Simulation smoke test</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Local machine</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>./scripts/smoke_test_main_simulation.py</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>4 dashboard nodes and 4 LoRa nodes</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>Terminal output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>Firmware build</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Local machine / PlatformIO</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>pio run in each firmware folder</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Build success</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>Build logs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>LoRa bench test</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Hardware bench</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Run sender + gateway + lora_gateway_serial.py</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>Packets stored in /api/lora/packets</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>RSSI/SNR/PDR logs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>Field test</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>Deployment site</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>Run Test Campaign T001-T010</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>Pass/fail per test</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>Workbook Test Campaign evidence</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Known Issues</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Open issues that affect workflow, validation, or deployment.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Issue</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Severity</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Impact</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Next Action</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>GitHub credential lacks workflow scope</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>CI workflow not pushed to GitHub</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Enable workflow scope or push CI with proper token/app.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>PlatformIO unavailable locally</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Firmware builds not locally validated</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>Install PlatformIO and run pio builds.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>Battery chemistry/Ah unknown</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Runtime and low-voltage thresholds uncertain</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>Confirm exact battery specs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>Real hardware not connected</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Expected</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>No field validation yet</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>Run deployment checklist when hardware is available.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Troubleshooting Logs</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Concise troubleshooting history and resolutions.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Problem</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Cause</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Resolution</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>GitHub push rejected for workflow file</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>HTTPS credential lacks workflow scope</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>Pushed code/workbook baseline without CI workflow; preserved CI locally</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Remote main b09c2c6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Initial GitHub repo had placeholder README</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>GitHub created README on repo creation</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Resolved by keeping full project README in pushed snapshot</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>README on remote project</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Local camera unavailable without OpenCV</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>cv2 missing on Mac venv</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Added PIL simulation fallback</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>/video_feed/0 smoke test</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Continuation Instructions</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>How to resume with minimum context and lowest capable model.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Step</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Action</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Recommended Tool</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Open workbook and read Active Context Snapshot + AI Session Handoff</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Any model</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>Current state summary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Check GitHub repo main and local branch status</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Local machine</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Confirm latest commit and dirty files</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Choose cheapest capable model using AI Router</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>ChatGPT/Roo</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Model/tool selection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Run local validation only when needed</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Local machine</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>Logs/screenshots</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>Use Codex only for focused repo execution/validation</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>Changed files + validation result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>Update workbook only after a major milestone/test/config change</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>Selected tool</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>Concise tracker/log rows</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Repo Structure</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Proposed GitHub repository layout.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Path</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Initial Source</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Living project reference</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Created by Codex</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>Created Locally</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>Commit once repo exists.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>docs/artifacts/</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>PDF/PNG/meeting references or summaries</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>User artifacts</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>Avoid committing huge video unless desired; store transcript/summary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>firmware/esp32-firenode/</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>ESP32 sensor + LoRa firmware</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>ESP/FireNode_ESP32_v5</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>PlatformIO project.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>raspi/firenode-system/</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>Main/node Flask app</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>RPi v4 ZIP</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>Created Locally</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>Refactor role-specific config.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>raspi/services/lora_gateway.py</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>Main LoRa receiver service</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>New</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>SPI or serial bridge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
+        <x:v>raspi/services/recorder.py</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>Camera event recording worker</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>New</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="str">
+        <x:v>ffmpeg/OpenCV.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="17" t="str">
+        <x:v>raspi/tests/</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="str">
+        <x:v>Unit/integration tests</x:v>
+      </x:c>
+      <x:c r="C11" s="17" t="str">
+        <x:v>New</x:v>
+      </x:c>
+      <x:c r="D11" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E11" s="17" t="str">
+        <x:v>Mock hardware where possible.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="17" t="str">
+        <x:v>.github/workflows/ci.yml</x:v>
+      </x:c>
+      <x:c r="B12" s="17" t="str">
+        <x:v>Python + PlatformIO CI</x:v>
+      </x:c>
+      <x:c r="C12" s="17" t="str">
+        <x:v>New</x:v>
+      </x:c>
+      <x:c r="D12" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E12" s="17" t="str">
+        <x:v>After repo exists.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="17" t="str">
+        <x:v>README.md</x:v>
+      </x:c>
+      <x:c r="B13" s="17" t="str">
+        <x:v>Project overview and run instructions</x:v>
+      </x:c>
+      <x:c r="C13" s="17" t="str">
+        <x:v>New</x:v>
+      </x:c>
+      <x:c r="D13" s="17" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E13" s="17" t="str">
+        <x:v>Should link workbook.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5552,6 +7350,649 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28.829999923706055" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21.469999313354492" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Change Log</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Chronological log of workbook/code changes.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Change ID</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>Summary</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Files / Sheets</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>Tests / Verification</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>Git Commit / PR</x:v>
+      </x:c>
+      <x:c r="H4" s="16" t="str">
+        <x:v>Next Step</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="17" t="str">
+        <x:v>C001</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>Workbook</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>Created ADM FireNode implementation workbook from reference format and all gathered FireNode requirements</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
+        <x:v>All workbook sheets</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="str">
+        <x:v>Workbook inspected/rendered locally</x:v>
+      </x:c>
+      <x:c r="G5" s="17" t="str">
+        <x:v>Pending GitHub repo</x:v>
+      </x:c>
+      <x:c r="H5" s="17" t="str">
+        <x:v>Provide repo/branch and commit workbook</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>C002</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Repository</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Initialized local Git repo, created clean baseline folders, imported RPi v4 app and ESP32 v5 firmware, added simulation start docs/script</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>.gitignore; README.md; raspi/; firmware/; simulation/; scripts/; docs/artifacts</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>python3 -m compileall -q raspi/firenode-system</x:v>
+      </x:c>
+      <x:c r="G6" s="17" t="str">
+        <x:v>21004de</x:v>
+      </x:c>
+      <x:c r="H6" s="17" t="str">
+        <x:v>Run simulation baseline and push after remote is provided</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="17" t="str">
+        <x:v>C003</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>Simulation</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>Verified main dashboard starts in simulation mode with one main node and three simulated remotes; updated start script to use local venv when present</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
+        <x:v>scripts/start_main_simulation.sh; raspi/firenode-system/config.json; Progress Tracker; Issue Log; Change Log</x:v>
+      </x:c>
+      <x:c r="F7" s="17" t="str">
+        <x:v>HTTP 200 /; /api/server-dashboard returned 4 nodes and 3 remotes</x:v>
+      </x:c>
+      <x:c r="G7" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H7" s="17" t="str">
+        <x:v>Implement cv2-free local camera simulation fallback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="17" t="str">
+        <x:v>C004</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>Simulation</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>Added cv2-free PIL fallback for the main node camera in simulation mode and suppressed macOS hostname warning</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str">
+        <x:v>modules/camera_stream.py; modules/network_utils.py; app.py; Progress Tracker; Issue Log; Change Log</x:v>
+      </x:c>
+      <x:c r="F8" s="17" t="str">
+        <x:v>compileall passed; /api/server-dashboard local camera running=true simulation=true; /video_feed/0 returned MJPEG</x:v>
+      </x:c>
+      <x:c r="G8" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H8" s="17" t="str">
+        <x:v>Implement LoRa packet simulation/receiver path</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="17" t="str">
+        <x:v>C005</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>LoRa Simulation</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>Added simulated LoRa receiver packet contract, dashboard fields, and API endpoint for RSSI/SNR/PDR/sequence/battery telemetry</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>modules/lora_simulator.py; app.py; static/app.js; simulation/README.md; scripts/start_main_simulation.sh; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F9" s="17" t="str">
+        <x:v>compileall passed; /api/lora/status active_nodes=4; /api/server-dashboard includes lora packet for main node</x:v>
+      </x:c>
+      <x:c r="G9" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H9" s="17" t="str">
+        <x:v>Implement real LoRa receiver adapter and SQLite packet store</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="17" t="str">
+        <x:v>C006</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>LoRa Storage</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>Added SQLite LoRa packet store plus /api/lora/packets and /api/lora/ingest so simulated and future hardware packets share persistence</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="str">
+        <x:v>modules/lora_packet_store.py; app.py; simulation/README.md; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="str">
+        <x:v>compileall passed; /api/lora/status stored_packet_count=8; /api/lora/packets returned rows</x:v>
+      </x:c>
+      <x:c r="G10" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H10" s="17" t="str">
+        <x:v>Implement real LoRa receiver adapter</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="17" t="str">
+        <x:v>C007</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C11" s="17" t="str">
+        <x:v>LoRa Gateway</x:v>
+      </x:c>
+      <x:c r="D11" s="17" t="str">
+        <x:v>Added serial gateway adapter for ESP32/SX127x JSON-line LoRa packets and documented first hardware bridge command</x:v>
+      </x:c>
+      <x:c r="E11" s="17" t="str">
+        <x:v>lora_gateway_serial.py; requirements.txt; simulation/README.md; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F11" s="17" t="str">
+        <x:v>compileall passed</x:v>
+      </x:c>
+      <x:c r="G11" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H11" s="17" t="str">
+        <x:v>Build ESP32 gateway firmware packet output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="17" t="str">
+        <x:v>C008</x:v>
+      </x:c>
+      <x:c r="B12" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C12" s="17" t="str">
+        <x:v>Firmware</x:v>
+      </x:c>
+      <x:c r="D12" s="17" t="str">
+        <x:v>Added dedicated ESP32 LoRa gateway firmware project that receives SX1278 packets, normalizes metadata, and emits one JSON packet per serial line</x:v>
+      </x:c>
+      <x:c r="E12" s="17" t="str">
+        <x:v>firmware/esp32-lora-gateway; lora_gateway_serial.py; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F12" s="17" t="str">
+        <x:v>Python parser smoke test passed; PlatformIO not installed locally, so firmware compile not run</x:v>
+      </x:c>
+      <x:c r="G12" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H12" s="17" t="str">
+        <x:v>Add automated tests for LoRa parser/store APIs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="17" t="str">
+        <x:v>C009</x:v>
+      </x:c>
+      <x:c r="B13" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C13" s="17" t="str">
+        <x:v>Tests</x:v>
+      </x:c>
+      <x:c r="D13" s="17" t="str">
+        <x:v>Added unittest coverage for LoRa serial parsing, SQLite packet dedupe/history, and simulator packet metrics</x:v>
+      </x:c>
+      <x:c r="E13" s="17" t="str">
+        <x:v>raspi/firenode-system/tests/test_lora_pipeline.py; scripts/run_raspi_tests.sh; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F13" s="17" t="str">
+        <x:v>./scripts/run_raspi_tests.sh: 4 tests OK</x:v>
+      </x:c>
+      <x:c r="G13" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H13" s="17" t="str">
+        <x:v>Implement camera recording on chainsaw event</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="17" t="str">
+        <x:v>C010</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C14" s="17" t="str">
+        <x:v>Recording</x:v>
+      </x:c>
+      <x:c r="D14" s="17" t="str">
+        <x:v>Added event recorder that saves chainsaw camera snapshots plus metadata and exposes /api/recordings</x:v>
+      </x:c>
+      <x:c r="E14" s="17" t="str">
+        <x:v>modules/event_recorder.py; app.py; tests/test_lora_pipeline.py; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F14" s="17" t="str">
+        <x:v>./scripts/run_raspi_tests.sh: 5 tests OK</x:v>
+      </x:c>
+      <x:c r="G14" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H14" s="17" t="str">
+        <x:v>Add dashboard recording list</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="17" t="str">
+        <x:v>C011</x:v>
+      </x:c>
+      <x:c r="B15" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C15" s="17" t="str">
+        <x:v>Dashboard</x:v>
+      </x:c>
+      <x:c r="D15" s="17" t="str">
+        <x:v>Added recent recordings panel and /media route so chainsaw snapshots can be reviewed in the web GUI</x:v>
+      </x:c>
+      <x:c r="E15" s="17" t="str">
+        <x:v>templates/dashboard.html; static/app.js; static/style.css; app.py; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F15" s="17" t="str">
+        <x:v>./scripts/run_raspi_tests.sh: 5 tests OK; / and /api/recordings returned 200</x:v>
+      </x:c>
+      <x:c r="G15" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H15" s="17" t="str">
+        <x:v>Add CI workflow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="17" t="str">
+        <x:v>C012</x:v>
+      </x:c>
+      <x:c r="B16" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C16" s="17" t="str">
+        <x:v>CI/CD</x:v>
+      </x:c>
+      <x:c r="D16" s="17" t="str">
+        <x:v>Added GitHub Actions workflow for Python app tests, compileall, and PlatformIO builds for sender and gateway firmware</x:v>
+      </x:c>
+      <x:c r="E16" s="17" t="str">
+        <x:v>.github/workflows/ci.yml; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F16" s="17" t="str">
+        <x:v>./scripts/run_raspi_tests.sh: 5 tests OK; PlatformIO unavailable locally</x:v>
+      </x:c>
+      <x:c r="G16" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H16" s="17" t="str">
+        <x:v>Add deployment/systemd scripts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="17" t="str">
+        <x:v>C013</x:v>
+      </x:c>
+      <x:c r="B17" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C17" s="17" t="str">
+        <x:v>Deployment</x:v>
+      </x:c>
+      <x:c r="D17" s="17" t="str">
+        <x:v>Added systemd install/stop scripts for the LoRa serial gateway bridge and documented gateway service operations</x:v>
+      </x:c>
+      <x:c r="E17" s="17" t="str">
+        <x:v>install_lora_gateway_service.sh; stop_lora_gateway_service.sh; README.md; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F17" s="17" t="str">
+        <x:v>bash -n scripts passed; ./scripts/run_raspi_tests.sh: 5 tests OK</x:v>
+      </x:c>
+      <x:c r="G17" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H17" s="17" t="str">
+        <x:v>Add API smoke-test script</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="17" t="str">
+        <x:v>C014</x:v>
+      </x:c>
+      <x:c r="B18" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C18" s="17" t="str">
+        <x:v>Testing</x:v>
+      </x:c>
+      <x:c r="D18" s="17" t="str">
+        <x:v>Added end-to-end simulation smoke test and wired it into CI</x:v>
+      </x:c>
+      <x:c r="E18" s="17" t="str">
+        <x:v>scripts/smoke_test_main_simulation.py; .github/workflows/ci.yml; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F18" s="17" t="str">
+        <x:v>./scripts/smoke_test_main_simulation.py passed</x:v>
+      </x:c>
+      <x:c r="G18" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H18" s="17" t="str">
+        <x:v>Add field deployment checklist/docs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="17" t="str">
+        <x:v>C015</x:v>
+      </x:c>
+      <x:c r="B19" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C19" s="17" t="str">
+        <x:v>Deployment</x:v>
+      </x:c>
+      <x:c r="D19" s="17" t="str">
+        <x:v>Added field deployment checklist covering bench prep, node install, LoRa validation, camera/recording checks, alert validation, and shutdown</x:v>
+      </x:c>
+      <x:c r="E19" s="17" t="str">
+        <x:v>docs/deployment/field_deployment_checklist.md; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F19" s="17" t="str">
+        <x:v>Documentation review</x:v>
+      </x:c>
+      <x:c r="G19" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H19" s="17" t="str">
+        <x:v>Add hardware wiring reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="17" t="str">
+        <x:v>C016</x:v>
+      </x:c>
+      <x:c r="B20" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C20" s="17" t="str">
+        <x:v>Hardware</x:v>
+      </x:c>
+      <x:c r="D20" s="17" t="str">
+        <x:v>Added wiring reference for ESP32 sensor sender, ESP32 LoRa gateway, main/remote Raspberry Pi devices, power notes, and open hardware decisions</x:v>
+      </x:c>
+      <x:c r="E20" s="17" t="str">
+        <x:v>docs/hardware/wiring_reference.md; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F20" s="17" t="str">
+        <x:v>Documentation review</x:v>
+      </x:c>
+      <x:c r="G20" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H20" s="17" t="str">
+        <x:v>Add README links to new docs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="17" t="str">
+        <x:v>C017</x:v>
+      </x:c>
+      <x:c r="B21" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C21" s="17" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="D21" s="17" t="str">
+        <x:v>Updated top-level README with fast start commands, current build path, and links to key project references</x:v>
+      </x:c>
+      <x:c r="E21" s="17" t="str">
+        <x:v>README.md; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F21" s="17" t="str">
+        <x:v>Documentation review</x:v>
+      </x:c>
+      <x:c r="G21" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H21" s="17" t="str">
+        <x:v>Add release/package script</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="17" t="str">
+        <x:v>C018</x:v>
+      </x:c>
+      <x:c r="B22" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C22" s="17" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="D22" s="17" t="str">
+        <x:v>Added release packaging script that uses git archive to create a clean zip under dist</x:v>
+      </x:c>
+      <x:c r="E22" s="17" t="str">
+        <x:v>scripts/package_release.sh; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F22" s="17" t="str">
+        <x:v>./scripts/package_release.sh produced dist zip</x:v>
+      </x:c>
+      <x:c r="G22" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H22" s="17" t="str">
+        <x:v>Add packet schema documentation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="17" t="str">
+        <x:v>C019</x:v>
+      </x:c>
+      <x:c r="B23" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C23" s="17" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="D23" s="17" t="str">
+        <x:v>Added LoRa sender payload, gateway serial line, ingest/history/status API, SQLite table, and validation target schema documentation</x:v>
+      </x:c>
+      <x:c r="E23" s="17" t="str">
+        <x:v>docs/api/lora_packet_schema.md; README.md; Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F23" s="17" t="str">
+        <x:v>Documentation review</x:v>
+      </x:c>
+      <x:c r="G23" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H23" s="17" t="str">
+        <x:v>Run full local verification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="17" t="str">
+        <x:v>C020</x:v>
+      </x:c>
+      <x:c r="B24" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C24" s="17" t="str">
+        <x:v>Verification</x:v>
+      </x:c>
+      <x:c r="D24" s="17" t="str">
+        <x:v>Completed full local verification checkpoint after unblocked development steps</x:v>
+      </x:c>
+      <x:c r="E24" s="17" t="str">
+        <x:v>Progress Tracker; Change Log</x:v>
+      </x:c>
+      <x:c r="F24" s="17" t="str">
+        <x:v>./scripts/run_raspi_tests.sh OK; ./scripts/smoke_test_main_simulation.py OK; python3 -m compileall OK; package_release produced dist/adm-firenode-192b1c7-20260514-141016.zip</x:v>
+      </x:c>
+      <x:c r="G24" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H24" s="17" t="str">
+        <x:v>Push to GitHub after remote is provided</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="17" t="str">
+        <x:v>C021</x:v>
+      </x:c>
+      <x:c r="B25" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C25" s="17" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="D25" s="17" t="str">
+        <x:v>Pushed project code, firmware, docs, and workbook to GitHub main; excluded CI workflow because token lacks workflow scope</x:v>
+      </x:c>
+      <x:c r="E25" s="17" t="str">
+        <x:v>Progress Tracker; Issue Log; GitHub Workflow; Change Log; workbook</x:v>
+      </x:c>
+      <x:c r="F25" s="17" t="str">
+        <x:v>git push to https://github.com/pagibetech/adm-firenode-forest-monitoring.git succeeded at commit 05e1a77</x:v>
+      </x:c>
+      <x:c r="G25" s="17" t="str">
+        <x:v>05e1a77 on GitHub</x:v>
+      </x:c>
+      <x:c r="H25" s="17" t="str">
+        <x:v>Enable workflow scope to push CI workflow later</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="17" t="str">
+        <x:v>C022</x:v>
+      </x:c>
+      <x:c r="B26" s="17" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="C26" s="17" t="str">
+        <x:v>AI Workflow</x:v>
+      </x:c>
+      <x:c r="D26" s="17" t="str">
+        <x:v>Added hybrid low-cost AI workflow workbook sheets for model routing, active context, handoff, validation matrix, environment, logs, and continuation</x:v>
+      </x:c>
+      <x:c r="E26" s="17" t="str">
+        <x:v>Active Context Snapshot; AI Session Handoff; AI Stack; AI Router; AI Model Routing Log; Codex Task Log; Build Validation Matrix; Environment Snapshot; Prompt Library</x:v>
+      </x:c>
+      <x:c r="F26" s="17" t="str">
+        <x:v>Workbook rendered and formula scan clean</x:v>
+      </x:c>
+      <x:c r="G26" s="17" t="str">
+        <x:v>Pending commit</x:v>
+      </x:c>
+      <x:c r="H26" s="17" t="str">
+        <x:v>Use workbook + GitHub as persistent project memory</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
Add Raspberry Pi deployment automation
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -1,48 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Architecture" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Phase Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Detailed Steps" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Hardware BOM" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Config Tracker" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Packet Protocol" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Backend APIs" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Database Schema" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Dashboard UX" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="AI &amp; Detection" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Camera &amp; Recording" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Deployment DevOps" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Test Campaign" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Progress Tracker" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Issue Log" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Decision Log" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Risk Register" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="System Diagram" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Data Flow" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Codex GitHub Workflow" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Codex Task Prompts" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Active Context Snapshot" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="AI Session Handoff" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Prompt Library" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Build Validation Matrix" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Environment Snapshot" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="AI Stack" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="AI Router" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="AI Model Routing Log" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="Codex Task Log" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="Software Dependencies" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="Simulation Plan" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="Validation Procedures" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="Known Issues" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="Troubleshooting Logs" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="Continuation Instructions" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="Repo Structure" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="Change Log" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Steps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardware BOM" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config Tracker" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packet Protocol" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend APIs" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database Schema" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard UX" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI &amp; Detection" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camera &amp; Recording" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment DevOps" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Campaign" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Tracker" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Log" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Diagram" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Flow" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex GitHub Workflow" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Task Prompts" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Context Snapshot" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Session Handoff" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Library" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Validation Matrix" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment Snapshot" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Stack" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Router" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Model Routing Log" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Task Log" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Software Dependencies" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulation Plan" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Procedures" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Issues" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Troubleshooting Logs" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuation Instructions" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo Structure" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -1979,7 +1979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -2275,6 +2275,70 @@
       <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Keep main/node config examples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Automated RPi deployment</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Use MacBook scripts to rsync app files, run setup, create venv, install requirements, write config, and create optional systemd service</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>All four RPis</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>Uses ~/admfire key, user betech, simulation mode, manual start default</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Manual start deployment mode</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Default behavior leaves service disabled; operator starts ./run.sh manually or enables service later</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>All four RPis</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_node.sh --install-service optional</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>Avoids surprise autostart during first hardware bench setup</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -3968,6 +4032,48 @@
       <c r="H31" s="17" t="inlineStr">
         <is>
           <t>Implement after simulation camera feeds are stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>P029</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Created MacBook-run automated Raspberry Pi deployment scripts for main server and three nodes in simulation mode</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>scripts/deploy_main_server.sh; scripts/deploy_node.sh; scripts/deploy_all_rpis.sh; docs/deployment/rpi_automated_deployment.md</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t>Run ./scripts/deploy_all_rpis.sh from MacBook when RPis are reachable</t>
         </is>
       </c>
     </row>
@@ -6445,7 +6551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -6692,6 +6798,40 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Current Milestone</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Automated Raspberry Pi deployment phase in simulation mode</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>ESP32/LoRa hardware validation paused; deploy RPis first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Next Recommended Action</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh from MacBook</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>Use SSH key ~/admfire and user betech against 192.168.9.51-.54.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6703,7 +6843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -6919,6 +7059,50 @@
       <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Avoid premium Codex for docs/simple edits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Unfinished: run automated RPi deployment</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Local machine / MacBook terminal</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh output, API responses, and stream placeholder checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Active assumption</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>ESP32/LoRa hardware validation paused</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>User instruction 2026-05-20</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Use simulation mode support on all RPis until hardware validation resumes</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -7405,6 +7589,43 @@
       <c r="G10" s="17" t="inlineStr">
         <is>
           <t>Need token with workflow scope; not blocking bench validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Automated Raspberry Pi deployment scripts</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Not yet run on RPis</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Ready for MacBook execution</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Shell syntax check passed</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>bash -n scripts/deploy_main_server.sh scripts/deploy_node.sh scripts/deploy_all_rpis.sh</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Needs live RPi deployment validation</t>
         </is>
       </c>
     </row>
@@ -8837,7 +9058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -9020,6 +9241,49 @@
           <t>b09c2c6 remote</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Create automated Raspberry Pi deployment scripts for simulation-mode deployment</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>/Users/macbookm1max321tb/A_Design/A_Coding/ADM Fire</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>scripts/deploy_main_server.sh; scripts/deploy_node.sh; scripts/deploy_all_rpis.sh; docs/deployment/rpi_automated_deployment.md; workflow memory docs; workbook</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>bash -n deployment scripts; deploy_node --help</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>Local script validation passed; live RPi deployment pending</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>ESP32/LoRa hardware validation paused; GitHub CI workflow scope issue may remain</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9494,7 +9758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -9696,6 +9960,114 @@
       <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Workbook Test Campaign evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Automated RPi script syntax</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>MacBook local repo</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>bash -n scripts/deploy_main_server.sh scripts/deploy_node.sh scripts/deploy_all_rpis.sh</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>No syntax errors</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Terminal output</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>RPi deployment execution</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>MacBook local repo</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>All four RPis receive app files, venv, config.json, and optional service file</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Terminal output and per-node deployment logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Simulation/API validation</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>MacBook after manual start</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>curl http://192.168.9.51:8090/api/status; curl http://192.168.9.51:8090/api/server-dashboard; curl http://192.168.9.52:8090/api/node-data</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Simulation mode API returns valid JSON and dashboard sees configured nodes</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Terminal output or screenshots</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Stream placeholder validation</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>MacBook after manual start</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>curl -I --max-time 5 http://192.168.9.51:8090/video_feed; curl --output /tmp/firenode-thermal.png http://192.168.9.51:8090/thermal.png</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Camera route responds and main thermal placeholder PNG is generated</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>Headers and PNG file output</t>
         </is>
       </c>
     </row>
@@ -10971,7 +11343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -11014,6 +11386,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -11977,6 +12350,48 @@
       <c r="H26" s="17" t="inlineStr">
         <is>
           <t>Use workbook + GitHub as persistent project memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>C023</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>Added MacBook-run automated deployment scripts for the four Raspberry Pis with simulation-mode config, optional systemd service, manual start default, and beginner validation guide</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>scripts/deploy_main_server.sh; scripts/deploy_node.sh; scripts/deploy_all_rpis.sh; docs/deployment/rpi_automated_deployment.md; workflow memory docs</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>bash -n passed; deploy_node --help checked</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>Pending commit</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t>Run deployment on live RPis and capture validation results</t>
         </is>
       </c>
     </row>
@@ -11991,7 +12406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -12034,6 +12449,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -12661,6 +13077,48 @@
         </is>
       </c>
       <c r="H19" s="17" t="str"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>S016</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Create automated Raspberry Pi deployment scripts using SSH key auth, simulation config, manual start default, and optional systemd service</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Hardware Bench Validation Phase / SSH key deployment complete</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>MacBook deployment scripts and beginner guide</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>bash -n passed for deployment scripts</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Improve Raspberry Pi deployment orchestration
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -2774,7 +2774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -4077,6 +4077,48 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>P030</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>Updated Raspberry Pi deployment scripts for parallel default, sequential mode, single-target deploy, per-IP logs, final pass/fail summary, and deployment role labels</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>bash -n passed; deploy_all help checked; Python tests and smoke test passed</t>
+        </is>
+      </c>
+      <c r="H33" s="17" t="inlineStr">
+        <is>
+          <t>Run ./scripts/deploy_all_rpis.sh from MacBook</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4088,7 +4130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -4131,6 +4173,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -4424,6 +4467,43 @@
       <c r="G11" s="17" t="inlineStr">
         <is>
           <t>Added PIL-based local camera fallback for simulation mode; live mode still uses OpenCV on Raspberry Pi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>I008</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>ESP32/SX1278 Hardware Validation Paused</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>ESP32 firmware builds/uploads, but real SX1278/Ra-02 validation is paused due to likely wiring or power instability</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Do not modify ESP32 firmware or start real LoRa integration during RPi simulation deployment phase</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>User/Codex</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>Proceed with Raspberry Pi simulation-mode deployment only; resume hardware validation after wiring/power is stabilized.</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -6832,6 +6912,40 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Next Incomplete Task</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh from MacBook</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>Parallel by default; use --sequential or --target &lt;ip&gt; if needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Paused Work</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>ESP32/SX1278 hardware validation paused</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>Likely wiring/power instability; do not modify firmware now.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6843,7 +6957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -7103,6 +7217,28 @@
       <c r="D13" s="17" t="inlineStr">
         <is>
           <t>Use simulation mode support on all RPis until hardware validation resumes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Next command</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Local MacBook terminal</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh; then inspect logs/deploy_*.log and validate dashboard/API</t>
         </is>
       </c>
     </row>
@@ -7290,7 +7426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -7624,6 +7760,43 @@
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Needs live RPi deployment validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Automated RPi deployment orchestration v2</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Not yet run on RPis</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Ready for MacBook execution</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Syntax/help/unit/smoke validation passed</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>bash -n; ./scripts/deploy_all_rpis.sh --help; ./scripts/run_raspi_tests.sh; ./scripts/smoke_test_main_simulation.py</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>Needs live RPi deployment validation</t>
         </is>
@@ -9058,7 +9231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -9284,6 +9457,49 @@
         </is>
       </c>
       <c r="I7" s="17" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Update RPi deployment scripts for parallel/sequential/targeted deployment and role labels</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>/Users/macbookm1max321tb/A_Design/A_Coding/ADM Fire</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>scripts/deploy_all_rpis.sh; scripts/deploy_node.sh; scripts/deploy_main_server.sh; raspi/firenode-system/app.py; docs/deployment/rpi_automated_deployment.md; workflow docs; workbook</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>bash -n; deploy_all --help; deploy_node --help; py_compile app.py; run_raspi_tests.sh; smoke_test_main_simulation.py</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>Passed locally; live RPi deployment pending</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>ESP32/SX1278 validation paused due wiring/power instability</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9758,7 +9974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -10068,6 +10284,87 @@
       <c r="E13" s="17" t="inlineStr">
         <is>
           <t>Headers and PNG file output</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Parallel RPi deployment</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>MacBook local repo</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>All four RPis deploy in parallel and logs are written under logs/deploy_&lt;ip&gt;.log</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>Final PASS/FAIL summary and per-IP logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Sequential RPi deployment</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>MacBook local repo</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh --sequential</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Each RPi deploys one at a time with per-IP logs</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Terminal output and logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Single target RPi deployment</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>MacBook local repo</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh --target 192.168.9.52</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Only selected RPi deploys and summary reports one target</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>Target log file</t>
         </is>
       </c>
     </row>
@@ -11343,7 +11640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -12392,6 +12689,48 @@
       <c r="H27" s="17" t="inlineStr">
         <is>
           <t>Run deployment on live RPis and capture validation results</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>C024</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>Updated RPi deployment automation for parallel default deployment, sequential mode, target-only mode, per-IP logs, pass/fail summary, and simulation role labels; recorded ESP32 hardware validation pause</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>scripts/deploy_all_rpis.sh; scripts/deploy_node.sh; scripts/deploy_main_server.sh; raspi/firenode-system/app.py; docs/deployment/rpi_automated_deployment.md; workflow docs; workbook</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>bash -n passed; help output checked; Python tests OK; smoke test OK</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>Pending commit</t>
+        </is>
+      </c>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
+          <t>Run ./scripts/deploy_all_rpis.sh from MacBook</t>
         </is>
       </c>
     </row>
@@ -12449,7 +12788,6 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Raspberry Pi USB camera capture
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -1733,7 +1733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -1965,6 +1965,38 @@
       <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Do not fill SD card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>USB camera capture format</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Live mode opens /dev/videoN with V4L2, applies MJPG FOURCC before size/FPS, discards warmup frames, and reopens on read failure</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>RPi dashboard live camera</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>/video_feed and /video_feed/&lt;index&gt;</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Implemented; pending RPi validation</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>Does not affect thermal stream or simulation mode.</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -4119,6 +4151,48 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>P031</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>Added configurable USB camera capture format for Raspberry Pi live mode after /dev/video0 required V4L2 + MJPG to read frames</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Done; pending RPi redeploy validation</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="G34" s="17" t="inlineStr">
+        <is>
+          <t>camera_stream.py; camera_test.py; config fields; docs/workbook/status updates</t>
+        </is>
+      </c>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh --target 192.168.9.51 --skip-setup</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4130,7 +4204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -4504,6 +4578,43 @@
       <c r="G12" s="17" t="inlineStr">
         <is>
           <t>Proceed with Raspberry Pi simulation-mode deployment only; resume hardware validation after wiring/power is stabilized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>I009</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Main Server USB Camera Frame Read Failed</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Main server dashboard/API work on 192.168.9.51, but /dev/video0 live camera reads failed with default OpenCV capture</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Dashboard camera panel unavailable until capture uses V4L2 + MJPG settings</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>User/Codex</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>Fixed in code; pending RPi redeploy/validation</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>Added configurable camera_backend, camera_fourcc, warmup frames, retry/reopen, and camera_test.py.</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -6946,6 +7057,40 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Current Issue</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Main server /dev/video0 needs V4L2 + MJPG capture settings</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Default OpenCV capture read failed; manual V4L2 MJPG test worked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Next Recommended Action</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh --target 192.168.9.51 --skip-setup</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>Then run camera_test.py and validate /video_feed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6957,7 +7102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -7239,6 +7384,28 @@
       <c r="D14" s="17" t="inlineStr">
         <is>
           <t>./scripts/deploy_all_rpis.sh; then inspect logs/deploy_*.log and validate dashboard/API</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Unfinished: validate main-server camera fix</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Local MacBook + Main RPi</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Targeted redeploy, camera_test.py output, /video_feed response, dashboard screenshot</t>
         </is>
       </c>
     </row>
@@ -7426,7 +7593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -7799,6 +7966,43 @@
       <c r="G12" s="17" t="inlineStr">
         <is>
           <t>Needs live RPi deployment validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB camera MJPG/V4L2 capture fix</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Pass local compile/tests</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Pending live RPi validation</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Ready for targeted main-server redeploy</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>py_compile, unit tests, smoke test, camera_test --help passed</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>python3 -m py_compile; ./scripts/run_raspi_tests.sh; ./scripts/smoke_test_main_simulation.py</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>Run camera_test.py and /video_feed check on 192.168.9.51</t>
         </is>
       </c>
     </row>
@@ -9231,7 +9435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -9500,6 +9704,49 @@
         </is>
       </c>
       <c r="I8" s="17" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Fix Raspberry Pi USB camera capture format for main-server /dev/video0</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>/Users/macbookm1max321tb/A_Design/A_Coding/ADM Fire</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>camera_stream.py; camera_test.py; config.json; app.py; README/deployment docs; workflow docs; workbook</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>py_compile; run_raspi_tests.sh; smoke_test_main_simulation.py; camera_test.py --help; bash -n deployment scripts</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>Passed locally; live RPi camera validation pending</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>ESP32/LoRa validation remains paused</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9974,7 +10221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -10365,6 +10612,60 @@
       <c r="E16" s="17" t="inlineStr">
         <is>
           <t>Target log file</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB camera MJPG/V4L2 test</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Main server RPi</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>./venv/bin/python camera_test.py --device 0 --fourcc MJPG --width 640 --height 480 --fps 25</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Camera test passed and saves /tmp/firenode_camera_test.jpg</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Terminal output and saved frame</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Dashboard live camera route</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>MacBook after main server restart</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>curl -I --max-time 5 http://192.168.9.51:8090/video_feed</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>HTTP response from MJPEG stream and no Camera frame read failed status</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>curl output and dashboard screenshot</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -12731,6 +13032,48 @@
       <c r="H28" s="17" t="inlineStr">
         <is>
           <t>Run ./scripts/deploy_all_rpis.sh from MacBook</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>C025</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>Added configurable USB camera capture settings for live Raspberry Pi cameras: V4L2 backend, MJPG FOURCC, warmup frames, retry/reopen on failed reads, and RPi camera_test.py helper</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>raspi/firenode-system/modules/camera_stream.py; raspi/firenode-system/camera_test.py; raspi/firenode-system/app.py; raspi/firenode-system/config.json; docs; workbook</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>py_compile passed; unit tests OK; smoke test OK; camera_test.py --help OK</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>Pending commit</t>
+        </is>
+      </c>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t>Deploy to main server and validate /dev/video0 live feed</t>
         </is>
       </c>
     </row>
@@ -14085,7 +14428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -14541,6 +14884,134 @@
       <c r="F16" s="17" t="inlineStr">
         <is>
           <t>Deployment in Philippines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>camera_backend</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>V4L2</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Main server manual test</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>Uses cv2.CAP_V4L2 on Linux/live mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>camera_fourcc</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>MJPG</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Main server manual test</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Applied before width/height/fps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>camera_open_warmup_frames</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Main server manual test</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Discard initial frames after opening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>camera_retry_on_failed_read</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Main server issue</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Release/reopen capture after failed read.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lower Raspberry Pi camera defaults
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -1733,7 +1733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -1997,6 +1997,38 @@
       <c r="F10" s="17" t="inlineStr">
         <is>
           <t>Does not affect thermal stream or simulation mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>RPi 3B camera stability defaults</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Use 320x240, 10 FPS, JPEG quality 55, MJPG, 10 warmup frames before trying higher settings</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Live USB camera</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>/video_feed and camera_test.py</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Updated; pending RPi validation</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>Corrupt MJPG frames can indicate USB bandwidth or camera power limits.</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -4193,6 +4225,48 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>P032</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>Lowered Raspberry Pi 3B USB camera defaults after corrupted MJPG frames at higher settings</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Done; pending RPi validation</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>app/config/static/deploy/docs/workbook updated</t>
+        </is>
+      </c>
+      <c r="H35" s="17" t="inlineStr">
+        <is>
+          <t>./scripts/deploy_all_rpis.sh --target 192.168.9.51 --skip-setup</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4204,7 +4278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -4247,7 +4321,6 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -4615,6 +4688,43 @@
       <c r="G13" s="17" t="inlineStr">
         <is>
           <t>Added configurable camera_backend, camera_fourcc, warmup frames, retry/reopen, and camera_test.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>I010</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>RPi 3B USB Camera Corrupt MJPG Frames</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>USB stream works but image is corrupted/unclear; manual MJPG test warned Corrupt JPEG data: premature end of data segment</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Dashboard image quality unstable at higher USB camera settings</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>User/Codex</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Mitigated in defaults; pending RPi validation</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>Lowered defaults to 320x240, 10 FPS, JPEG quality 55, MJPG, 10 warmup frames.</t>
         </is>
       </c>
     </row>
@@ -6742,7 +6852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -7091,6 +7201,23 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Camera Stability Default</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>320x240, 10 FPS, JPEG quality 55, MJPG, 10 warmup frames</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Use lower settings first on RPi 3B due possible USB bandwidth/power limit.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7102,7 +7229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -7406,6 +7533,28 @@
       <c r="D15" s="17" t="inlineStr">
         <is>
           <t>Targeted redeploy, camera_test.py output, /video_feed response, dashboard screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Unfinished: validate low-bandwidth camera defaults</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Local MacBook + Main RPi</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Deploy to 192.168.9.51, run camera_test.py at 320x240/10 FPS, inspect dashboard image clarity</t>
         </is>
       </c>
     </row>
@@ -7593,7 +7742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -8003,6 +8152,43 @@
       <c r="G13" s="17" t="inlineStr">
         <is>
           <t>Run camera_test.py and /video_feed check on 192.168.9.51</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>RPi 3B camera stability defaults</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Pass local compile/tests</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Pending live RPi validation</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Ready for targeted main-server redeploy</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>py_compile, unit tests, smoke test, camera_test --help, and deploy script syntax passed locally</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>py_compile; unit tests; smoke test; camera_test --help</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>Run low-bandwidth camera_test on 192.168.9.51</t>
         </is>
       </c>
     </row>
@@ -9435,7 +9621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -9747,6 +9933,49 @@
         </is>
       </c>
       <c r="I9" s="17" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Lower RPi 3B USB camera defaults for stability</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>/Users/macbookm1max321tb/A_Design/A_Coding/ADM Fire</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>camera defaults/config/docs/workbook</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>py_compile; run_raspi_tests.sh; smoke_test_main_simulation.py; camera_test.py --help; bash -n deploy scripts</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>Passed locally; live RPi validation pending</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>Live RPi validation required</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I10" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10221,7 +10450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -10666,6 +10895,33 @@
       <c r="E18" s="17" t="inlineStr">
         <is>
           <t>curl output and dashboard screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>RPi 3B low-bandwidth USB camera test</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Main server RPi</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>./venv/bin/python camera_test.py --device 0 --fourcc MJPG --width 320 --height 240 --fps 10</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Camera test passes without corrupt/unclear image</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Terminal output and /tmp/firenode_camera_test.jpg</t>
         </is>
       </c>
     </row>
@@ -11941,7 +12197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -11984,7 +12240,6 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -13074,6 +13329,48 @@
       <c r="H29" s="17" t="inlineStr">
         <is>
           <t>Deploy to main server and validate /dev/video0 live feed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>C026</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Lowered RPi 3B USB camera defaults to 320x240, 10 FPS, JPEG quality 55, MJPG, and 10 warmup frames after corrupt MJPG frame warnings</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>app.py; config.json; camera_stream.py; camera_test.py; static/app.js; docs; workbook</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>py_compile passed; unit tests OK; smoke test OK; camera_test.py --help OK; deploy scripts syntax OK</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>Pending commit</t>
+        </is>
+      </c>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t>Deploy to main server and validate image clarity</t>
         </is>
       </c>
     </row>
@@ -14428,7 +14725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -15012,6 +15309,198 @@
       <c r="F20" s="17" t="inlineStr">
         <is>
           <t>Release/reopen capture after failed read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>camera_width</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Main server camera stability finding</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>Lower default for Raspberry Pi 3B USB stability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>camera_height</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Main server camera stability finding</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>Lower default for Raspberry Pi 3B USB stability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>camera_fps</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Main server camera stability finding</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>Reduced FPS to limit USB bandwidth/power stress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>camera_jpeg_quality</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>Main server camera stability finding</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>Reduced JPEG quality for smaller MJPEG stream frames.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>camera_fourcc</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>MJPG</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Main server camera stability finding</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>Keep MJPG as confirmed working format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>camera_open_warmup_frames</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>RPi USB cameras</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Main server camera stability finding</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Discard more startup frames before streaming.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update FireNode CSI camera validation status
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -2478,7 +2478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -2521,6 +2521,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -2925,7 +2926,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>.51/.52 confirmed</t>
+          <t>.51/.52/.53/.54 confirmed</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3037,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>.51/.52 confirmed</t>
+          <t>.51/.52/.53/.54 confirmed</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3074,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>rpicam-still confirmed on .51/.52</t>
+          <t>rpicam-still confirmed on .51/.52/.53/.54</t>
         </is>
       </c>
     </row>
@@ -3105,12 +3106,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>modules implemented; pending deploy to .51/.52</t>
+          <t>modules implemented and deployed to .51/.52/.53/.54; /video_feed validated</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3333,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Code implemented; pending deployment and live validation. DO NOT MARK PASS YET.</t>
+          <t>Code implemented; pending .51 availability for deployment and live validation. DO NOT MARK PASS YET.</t>
         </is>
       </c>
     </row>
@@ -3364,12 +3365,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>CSI cameras installed; remaining components pending assembly.</t>
+          <t>CSI cameras installed and validated on .53/.54; ESP32 + LoRa + sensors pending assembly.</t>
         </is>
       </c>
     </row>
@@ -3444,6 +3445,154 @@
       <c r="G29" t="inlineStr">
         <is>
           <t>Synthetic test audio exists; live microphone pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>T031</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CSI camera validation .53</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Open NODE_02 dashboard in LIVE mode and verify local camera feed</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Clear MJPEG stream from .53 CSI camera at configured resolution/FPS</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Stream stability</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Visual inspection; rpicam-hello confirmed ov5647 on .53; required python3-picamera2 and file sync</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>T032</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CSI camera validation .54</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Open NODE_03 dashboard in LIVE mode and verify local camera feed</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Clear MJPEG stream from .54 CSI camera at configured resolution/FPS</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Stream stability</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Visual inspection; rpicam-hello confirmed ov5647 on .54; required python3-picamera2 and sync of modules/multi_camera_stream.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>T033</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>python3-picamera2 dependency check</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Run dpkg -s python3-picamera2 on .53 and .54</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Package is installed</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Dependency presence</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>sudo apt install -y python3-picamera2 executed on .53/.54</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>T034</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Deployment sync checklist .53/.54</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Verify app.py, static/app.js, templates/dashboard.html, modules/csi_camera_stream.py, modules/multi_camera_stream.py, config.json, .deployment.env</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Files synced and node-specific configs correct</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Deployment accuracy</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>NODE_02 required all listed files; NODE_03 required app.py, static/app.js, modules/csi_camera_stream.py, modules/multi_camera_stream.py, config</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -5199,7 +5348,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -5214,12 +5363,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Hardware installed; awaiting rpicam-hello confirmation</t>
+          <t>rpicam-hello confirmed ov5647 on .53; python3-picamera2 installed; file sync completed; local dashboard stream validated.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Run rpicam-hello --list-cameras on .53</t>
+          <t>ESP32 hardware assembly for NODE_02</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5390,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -5256,12 +5405,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Hardware installed; awaiting rpicam-hello confirmation</t>
+          <t>rpicam-hello confirmed ov5647 on .54; python3-picamera2 installed; modules/multi_camera_stream.py synced from NODE_01; local dashboard stream validated.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Run rpicam-hello --list-cameras on .54</t>
+          <t>ESP32 hardware assembly for NODE_03</t>
         </is>
       </c>
     </row>
@@ -5446,7 +5595,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -5461,12 +5610,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Hardware installed; awaiting rpicam-hello confirmation</t>
+          <t>rpicam-hello confirmed ov5647 on .53; python3-picamera2 installed; file sync completed; local dashboard stream validated.</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Run rpicam-hello --list-cameras on .53</t>
+          <t>ESP32 hardware assembly for NODE_02</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5637,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -5503,12 +5652,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Hardware installed; awaiting rpicam-hello confirmation</t>
+          <t>rpicam-hello confirmed ov5647 on .54; python3-picamera2 installed; modules/multi_camera_stream.py synced from NODE_01; local dashboard stream validated.</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Run rpicam-hello --list-cameras on .54</t>
+          <t>ESP32 hardware assembly for NODE_03</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5679,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -5540,17 +5689,17 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>modules/csi_camera_stream.py created; multi_camera_stream.py updated; app.py/config updated; py_compile passed</t>
+          <t>modules/csi_camera_stream.py created; multi_camera_stream.py updated; app.py/config updated; py_compile passed; deployed and validated on .51/.52/.53/.54</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Deploy to .51/.52 and validate /video_feed endpoint</t>
+          <t>Verify MAIN ESP32 serial integration when .51 is reachable</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5931,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -5797,7 +5946,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>CSI cameras installed; ESP32 hardware not yet assembled; no power/LoRa validation possible</t>
+          <t>CSI cameras installed and validated on .53/.54; ESP32 hardware not yet assembled; no power/LoRa validation possible</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -5887,6 +6036,132 @@
       <c r="H59" t="inlineStr">
         <is>
           <t>Install USB microphone on a node, run detector.py, and validate chainsaw alert + recording</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>P062</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CSI camera validation .53 PASS</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>User/Codex</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>NODE_02 .53 dashboard in LIVE mode; CSI camera feed clear and stable; python3-picamera2 installed</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Validate ESP32 hardware assembly for NODE_02</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>P063</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CSI camera validation .54 PASS</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>User/Codex</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>NODE_03 .54 dashboard in LIVE mode; CSI camera feed clear and stable; python3-picamera2 installed; modules/multi_camera_stream.py synced from NODE_01</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Validate ESP32 hardware assembly for NODE_03</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>P064</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>MAIN ESP32 USB serial reader PENDING VERIFICATION (blocked by .51 unavailability)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>modules/esp32_serial_reader.py created; app.py/config updated; py_compile passed; manual Minicom confirmed /dev/ttyUSB0 at 115200; .51 unreachable for live validation</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Deploy to .51 MAIN and validate live sensor cards from serial cache when .51 is reachable</t>
         </is>
       </c>
     </row>
@@ -5944,6 +6219,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -6616,7 +6892,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Deploy updated raspi/firenode-system to .51 and verify /api/status serial_connected=true and sensor cards populate from serial cache.</t>
+          <t>Code deployed to .51; LIVE dashboard sensor-card population from serial cache NOT YET VERIFIED. Blocked by .51 unavailability.</t>
         </is>
       </c>
     </row>
@@ -6653,7 +6929,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Assemble NODE_02/NODE_03 using NODE_01 wiring/firmware baseline; run rpicam-hello and LoRa bench test.</t>
+          <t>Assemble NODE_02/NODE_03 using NODE_01 baseline; run LoRa bench test. RPi CSI cameras are already operational.</t>
         </is>
       </c>
     </row>
@@ -9232,12 +9508,12 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>MAIN .51 dashboard LIVE mode; CSI cameras validated on .51/.52; remote node aggregation .51→.52 PASS; ESP32 serial reader implemented; minicom confirmed hardware.</t>
+          <t>MAIN .51 dashboard LIVE mode; CSI cameras validated on .51/.52/.53/.54; remote node aggregation .51→.52 PASS; ESP32 serial reader implemented; minicom confirmed hardware; NODE_02/NODE_03 CSI alignment completed.</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -9249,12 +9525,12 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>ESP32 Serial Reader Deployment Verification Phase</t>
+          <t>MAIN ESP32 USB serial integration verification (pending .51 availability)</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>Next: deploy to .51 and validate live sensor cards from serial.</t>
+          <t>Next: resume when .51 is reachable and validate live sensor cards from serial.</t>
         </is>
       </c>
     </row>
@@ -9266,12 +9542,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>CSI camera pipeline LIVE on .51/.52; ESP32 serial integration implemented pending verification</t>
+          <t>CSI camera pipeline LIVE on .51/.52/.53/.54; ESP32 serial integration implemented pending .51 verification</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>No new features until serial and remaining hardware are validated.</t>
+          <t>No new features until serial validation resumes and remaining hardware are validated.</t>
         </is>
       </c>
     </row>
@@ -9283,12 +9559,12 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>MAIN ESP32 dashboard live sensor integration pending verification; .53/.54 hardware build pending; thermal and audio pending hardware.</t>
+          <t>MAIN ESP32 dashboard live sensor integration pending verification (blocked by .51 unavailability); NODE_02/NODE_03 ESP32 hardware build pending; thermal and audio pending hardware.</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>Serial code is complete; deploy and confirm.</t>
+          <t>Serial code is complete; NODE_02/NODE_03 CSI cameras are operational.</t>
         </is>
       </c>
     </row>
@@ -9300,12 +9576,12 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>CSI camera .51/.52 PASS; remote aggregation PASS; serial hardware PASS; serial dashboard integration IN PROGRESS.</t>
+          <t>CSI camera .51/.52/.53/.54 PASS; remote aggregation PASS; serial hardware PASS; serial dashboard integration PENDING (blocked by .51 unavailability).</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Pending: deploy serial reader to .51 and confirm sensor card population.</t>
+          <t>Pending: .51 availability to deploy serial reader and confirm sensor card population.</t>
         </is>
       </c>
     </row>
@@ -9334,12 +9610,12 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Hardware bench validation extended: MAIN + NODE_01 camera and network validated; serial code ready</t>
+          <t>Hardware bench validation extended: MAIN + NODE_01 camera and network validated; NODE_02/NODE_03 CSI cameras validated; serial code ready</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>Focus on .51 deployment and sensor verification.</t>
+          <t>Focus on .51 availability and sensor verification.</t>
         </is>
       </c>
     </row>
@@ -9351,7 +9627,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Deploy updated raspi/firenode-system to .51 MAIN and validate live mode sensor cards from serial cache</t>
+          <t>Resume when MAIN .51 is reachable: deploy updated raspi/firenode-system and validate live mode sensor cards from serial cache</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
@@ -9368,7 +9644,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Deploy and verify ESP32 serial reader on .51 MAIN</t>
+          <t>Verify MAIN ESP32 USB serial integration on .51 MAIN (blocked by .51 unavailability)</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
@@ -9402,12 +9678,12 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>MAIN ESP32 serial integration implemented but not yet verified in live mode</t>
+          <t>MAIN ESP32 serial integration implemented but not yet verified in live mode (blocked by .51 unavailability)</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>Code complete; minicom confirmed hardware output; deployment pending.</t>
+          <t>Code complete; minicom confirmed hardware output; NODE_02/NODE_03 CSI cameras operational.</t>
         </is>
       </c>
     </row>
@@ -9419,7 +9695,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Deploy updated raspi/firenode-system to .51 MAIN and validate live mode sensor cards from serial cache</t>
+          <t>Resume when MAIN .51 is reachable: deploy updated raspi/firenode-system and validate live mode sensor cards from serial cache</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -9441,7 +9717,7 @@
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>CSI validated on .51/.52 in LIVE mode.</t>
+          <t>CSI validated on .51/.52/.53/.54 in LIVE mode.</t>
         </is>
       </c>
     </row>
@@ -9573,7 +9849,7 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
@@ -9683,12 +9959,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>NODE_02/NODE_03 CSI cameras validated; MAIN ESP32 serial pending .51 availability</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>Local machine / MacBook terminal</t>
+          <t>Selected AI/tool</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
@@ -9705,12 +9981,12 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>ESP32/LoRa hardware validation paused</t>
+          <t>Local machine first; Kimi for heavy implementation; Codex for repo execution/validation</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>User instruction 2026-05-20</t>
+          <t>AI Router</t>
         </is>
       </c>
       <c r="D13" s="17" t="inlineStr">
@@ -9727,12 +10003,12 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Local MacBook terminal</t>
+          <t>Local machine / MacBook terminal</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
@@ -9749,7 +10025,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>NODE_02/NODE_03 CSI validated; MAIN camera fix validated; low-bandwidth defaults no longer needed (CSI)</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
@@ -9771,7 +10047,7 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed (CSI replaces USB)</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
@@ -9969,7 +10245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -10012,6 +10288,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -10506,17 +10783,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pass on .51/.52</t>
+          <t>Pass on .51/.52/.53/.54</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Pending pipeline implementation</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ov5647 detected; rpicam-hello confirmed</t>
+          <t>ov5647 detected on .51/.52/.53/.54; rpicam-hello confirmed</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -10526,7 +10803,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Implement rpicam/libcamera capture module and integrate into camera_stream.py.</t>
+          <t>Detection confirmed on all nodes.</t>
         </is>
       </c>
     </row>
@@ -10617,7 +10894,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pass on .51/.52</t>
+          <t>Pass on .51/.52/.53/.54</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -10627,7 +10904,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ov5647 detected; rpicam-hello confirmed</t>
+          <t>ov5647 detected on .51/.52/.53/.54; rpicam-hello confirmed</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -10637,7 +10914,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Detection confirmed. Pipeline module implemented; pending deploy validation.</t>
+          <t>Detection confirmed on all nodes.</t>
         </is>
       </c>
     </row>
@@ -10654,17 +10931,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pending deploy validation on .51/.52</t>
+          <t>Pass on .51/.52/.53/.54</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>modules/csi_camera_stream.py + multi_camera_stream.py + app.py updates; py_compile passed</t>
+          <t>modules/csi_camera_stream.py + multi_camera_stream.py + app.py updates; py_compile passed; validated on all nodes</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -10971,6 +11248,191 @@
       <c r="G29" t="inlineStr">
         <is>
           <t>Deferred until USB microphone is installed on a node.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Raspberry Pi CSI camera pipeline (Picamera2)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Pass local compile/tests</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Pass on .51/.52/.53/.54</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>modules/csi_camera_stream.py + multi_camera_stream.py + app.py updates; py_compile passed; validated on all nodes</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>python3 -m py_compile; deploy to .51/.52/.53/.54; curl /video_feed</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>CSI primary with USB fallback; simulation preserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CSI camera validation .53</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>N/A (hardware)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Pass on .53</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>NODE_02 .53 dashboard in LIVE mode; CSI feed clear and stable</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Visual inspection on dashboard; rpicam-hello --list-cameras; curl /video_feed</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Required python3-picamera2 and file sync.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CSI camera validation .54</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>N/A (hardware)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Pass on .54</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>NODE_03 .54 dashboard in LIVE mode; CSI feed clear and stable</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Visual inspection on dashboard; rpicam-hello --list-cameras; curl /video_feed</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Required python3-picamera2 and sync of modules/multi_camera_stream.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>python3-picamera2 package dependency</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Required on .53/.54</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>sudo apt install -y python3-picamera2</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>dpkg -s python3-picamera2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Not preinstalled on fresh RPi OS Lite; required for Picamera2 CSI stream.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Deployment sync checklist (CSI alignment)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Required for .53/.54</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>app.py, static/app.js, templates/dashboard.html, modules/csi_camera_stream.py, modules/multi_camera_stream.py, config.json, .deployment.env</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>rsync / deploy scripts</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Ensure node-specific config values (name, IP, role) are correct per node.</t>
         </is>
       </c>
     </row>
@@ -12770,7 +13232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -13002,6 +13464,38 @@
       <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Used only for workbook generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Raspberry Pi CSI camera</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>python3-picamera2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Latest available via apt</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Required on .53/.54; confirmed installed</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>sudo apt install -y python3-picamera2</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Not preinstalled on RPi OS Lite; required for Picamera2 CSI stream.</t>
         </is>
       </c>
     </row>
@@ -13761,6 +14255,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -14012,22 +14507,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Cannot confirm ov5647 detection on NODE_02/NODE_03 until hardware is cabled and powered</t>
+          <t>ov5647 detection confirmed on .53/.54; local dashboard streams validated.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Run rpicam-hello --list-cameras on .53 and .54.</t>
+          <t>Complete.</t>
         </is>
       </c>
     </row>
@@ -14039,22 +14534,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Cannot confirm ov5647 detection on NODE_02/NODE_03 until hardware is cabled and powered</t>
+          <t>ov5647 detection confirmed on .53/.54; local dashboard streams validated.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Run rpicam-hello --list-cameras on .53 and .54.</t>
+          <t>Complete.</t>
         </is>
       </c>
     </row>
@@ -14076,12 +14571,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sensor cards on MAIN dashboard may still show HTTP fallback data instead of serial cache until deployment validation is complete</t>
+          <t>Sensor cards on MAIN dashboard may still show HTTP fallback data instead of serial cache until .51 is reachable and deployment validation is complete</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Deploy to .51 and verify /api/status serial_connected=true and sensor card values match minicom packets.</t>
+          <t>Resume when .51 is reachable: deploy and verify /api/status serial_connected=true and sensor card values match minicom packets.</t>
         </is>
       </c>
     </row>
@@ -14103,12 +14598,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cannot validate full 4-node mesh or complete camera grid until NODE_02/NODE_03 are assembled</t>
+          <t>Cannot validate full 4-node mesh or complete ESP32 sensor integration until NODE_02/NODE_03 are assembled. RPi CSI cameras are already operational.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Assemble using NODE_01 baseline; run LoRa bench test and rpicam-hello confirmation.</t>
+          <t>Assemble using NODE_01 baseline; run LoRa bench test.</t>
         </is>
       </c>
     </row>
@@ -15249,7 +15744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -17095,6 +17590,48 @@
       <c r="H46" s="18" t="inlineStr">
         <is>
           <t>Complete serial dashboard integration verification on .51; do NOT mark serial dashboard as PASS yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>C049</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>NODE_02 (.53) and NODE_03 (.54) CSI camera setup and validation completed</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>docs/ACTIVE_CONTEXT.md; docs/PROJECT_STATUS.md; docs/AI_SESSION_HANDOFF.md; docs/deployment/field_deployment_checklist.md; docs/ROO_HANDOFF_PROMPT.md; workbook</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Visual inspection on .53/.54 dashboards; rpicam-hello --list-cameras; curl /video_feed; /api/node-data camera_type=csi</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Pending commit</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Resume MAIN ESP32 serial verification when .51 is reachable</t>
         </is>
       </c>
     </row>
@@ -17176,12 +17713,12 @@
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>CSI CAMERA VALIDATED</t>
         </is>
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>Dashboard running in LIVE mode; local sensors, remote nodes, ESP32 serial all configured.</t>
+          <t>CSI cameras physically mounted and operational on .53/.54; live stream confirmed on local dashboards; ESP32 + LoRa + sensor modules not yet assembled.</t>
         </is>
       </c>
     </row>
@@ -17387,76 +17924,76 @@
     </row>
     <row r="14">
       <c r="A14" s="18" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Camera</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>ESP32 serial reader implementation</t>
+          <t>NODE_02 .53 CSI camera</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>IMPLEMENTED</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>modules/esp32_serial_reader.py created; py_compile + parse_line unit test passed.</t>
+          <t>ov5647 CSI camera confirmed via rpicam-hello; clear and stable feed on local dashboard; required python3-picamera2 and file sync.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Camera</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Serial dashboard integration</t>
+          <t>NODE_03 .54 CSI camera</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>PENDING VERIFICATION</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>Code deployed to .51; LIVE sensor-card population from serial cache NOT YET VERIFIED.</t>
+          <t>ov5647 CSI camera confirmed via rpicam-hello; clear and stable feed on local dashboard; required python3-picamera2 and sync of modules/multi_camera_stream.py from NODE_01.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="18" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>ESP32 sensor-sender firmware</t>
+          <t>Serial dashboard integration</t>
         </is>
       </c>
       <c r="D16" s="22" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PENDING VERIFICATION</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
         <is>
-          <t>DHT22/PIR/MQ/LoRa TX validated on MAIN and NODE_01 bench; NODE_02/03 pending.</t>
+          <t>Code deployed to .51; LIVE sensor-card population from serial cache NOT YET VERIFIED. Blocked by .51 unavailability.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add separate node dashboard gui
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -569,7 +569,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Next: Deploy updated raspi/firenode-system to .51 MAIN and validate live mode sensor cards from serial. Confirm NODE_01 camera remains visible on MAIN dashboard after redeploy. Assemble and validate .53/.54 hardware when available. Install thermal camera on MAIN when hardware arrives. Install USB microphone and validate chainsaw detection pipeline.</t>
+          <t>Separate NODE GUI implemented: node_dashboard.html + node_app.js for NODE RPis only (192.168.9.52/.53/.54). NODE GUI is one-page only with local camera, sensor readings, chainsaw controls/status, alerts, recordings. MAIN server dashboard (dashboard.html + app.js) preserved unchanged. NODE simulation mode forced to live. Chainsaw controls moved to NODE dashboard. No ESP32/LoRa/thermal architecture changes.</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,6 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -3607,7 +3606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -6162,6 +6161,132 @@
       <c r="H62" t="inlineStr">
         <is>
           <t>Deploy to .51 MAIN and validate live sensor cards from serial cache when .51 is reachable</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>P046</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Create separate one-page web GUI for NODE RPis only</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>node_dashboard.html and node_app.js created; app.py routes node role to node_dashboard.html</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Deploy to .52/.53/.54 and verify NODE GUI loads correctly</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>P047</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Move chainsaw controls to NODE dashboard page</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Chainsaw start/stop, sensitivity settings, audio test browser in node_dashboard.html</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Deploy and verify chainsaw detection from NODE GUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>P048</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Disable simulation mode for NODE RPis</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>operation_mode() forced to live when current_role() == node; simulation UI removed from NODE GUI</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Deploy and verify NODE-only live mode on .52/.53/.54</t>
         </is>
       </c>
     </row>
@@ -6219,7 +6344,6 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -7018,7 +7142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -7506,6 +7630,38 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>Install thermal on MAIN first; install USB mic on one node for chainsaw validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>D010</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Separate NODE GUI vs shared dashboard.html</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>NODE RPis need a simplified one-page dashboard without server-specific cards; MAIN dashboard must remain full-featured</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Maintainability and role-appropriate UX</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>app.py index() routes by role; node_dashboard.html is one-page; dashboard.html unchanged for MAIN</t>
         </is>
       </c>
     </row>
@@ -10245,7 +10401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -10288,7 +10444,6 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -11433,6 +11588,43 @@
       <c r="G34" t="inlineStr">
         <is>
           <t>Ensure node-specific config values (name, IP, role) are correct per node.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Node dashboard (node_dashboard.html + node_app.js)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Pass local py_compile and role routing logic</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Pending deployment to .52/.53/.54</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>templates/node_dashboard.html, static/node_app.js; app.py updated</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>python3 -m py_compile app.py modules/*.py</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>One-page NODE GUI with camera, sensors, chainsaw, alerts, recordings.</t>
         </is>
       </c>
     </row>
@@ -14255,7 +14447,6 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: sync workbook and docs with firmware + detection v2 state
Workbook sync (scripts/sync_workbook.py):
- Dashboard: updated current stage and next action
- Progress Tracker: +6 steps (P033-P038) for NODE dashboard,
  chainsaw UX, sample rate fix, device enum v2, NODE03 UART,
  multi-node firmware
- Active Context Snapshot: updated milestone, testing, next task
- Known Issues: updated I020 (USB mic/chainsaw)
- Change Log: +6 entries (C029-C034)
- Serial Update sheet: +5 status rows (17-21)

Documentation sync:
- ACTIVE_CONTEXT.md: firmware multi-env builds documented
- PROJECT_STATUS.md: firmware and detection v2 status
- AI_SESSION_HANDOFF.md: updated recent commits and handoff
</commit_message>
<xml_diff>
--- a/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
+++ b/docs/workbook/ADM_FireNode_Implementation_Workbook.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -569,10 +569,11 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Separate NODE GUI implemented: node_dashboard.html + node_app.js for NODE RPis only (192.168.9.52/.53/.54). NODE GUI is one-page only with local camera, sensor readings, chainsaw controls/status, alerts, recordings. MAIN server dashboard (dashboard.html + app.js) preserved unchanged. NODE simulation mode forced to live. Chainsaw controls moved to NODE dashboard. No ESP32/LoRa/thermal architecture changes.</t>
-        </is>
-      </c>
-    </row>
+          <t>NODE_03 UART wiring (when hardware available). Deploy updated node_app to .54. Verify NODE01/NODE02 UART readiness. Update workbook to reflect all implemented features. Commits: 423fb63 (device enum v2), daf78c4 (multi-node firmware).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -881,6 +882,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3606,7 +3608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -6287,6 +6289,258 @@
       <c r="H65" t="inlineStr">
         <is>
           <t>Deploy and verify NODE-only live mode on .52/.53/.54</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>P033</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Separate NODE dashboard (node_dashboard.html + node_app.js) for NODE RPis only; MAIN dashboard preserved</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>node_dashboard.html; node_app.js; app.py role routing</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>NODE GUI cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>P034</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Chainsaw detector UX: device selection, error visibility, Starting feedback, audio visualizer</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>app.py; detector.py; node_app.js</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Field validation with real mic</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>P035</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Sample rate fix: detector uses device default_samplerate instead of hardcoded 16000 Hz</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>detector.py _loop() updated</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Verify on all USB mic models</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>P036</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Live device enumeration v2: arecord -l non-zero exit authoritative (no stale PortAudio)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>app.py; tests/test_api_devices.py</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Field validate on RPi</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>P037</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>NODE03 (.54) UART readiness verified: /dev/serial0, serial reader connected</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>API local_serial.connected=true</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Wire ESP32 to GPIO UART</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>P038</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Firmware</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Multi-node firmware builds: 4 PlatformIO environments (main/node_01/node_02/node_03)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>4 firmware.bin files built; correct NODE_ID</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Flash when ESP32 hardware arrives</t>
         </is>
       </c>
     </row>
@@ -9554,6 +9808,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -9664,7 +9919,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>MAIN .51 dashboard LIVE mode; CSI cameras validated on .51/.52/.53/.54; remote node aggregation .51→.52 PASS; ESP32 serial reader implemented; minicom confirmed hardware; NODE_02/NODE_03 CSI alignment completed.</t>
+          <t>Multi-node firmware builds; live device enumeration v2 fix; NODE03 UART readiness verified. Commits: 423fb63, daf78c4.</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
@@ -9681,7 +9936,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>MAIN ESP32 USB serial integration verification (pending .51 availability)</t>
+          <t>NODE03 UART physical wiring (pending hardware); MAIN .51 serial validation (pending .51 availability)</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
@@ -9715,7 +9970,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>MAIN ESP32 dashboard live sensor integration pending verification (blocked by .51 unavailability); NODE_02/NODE_03 ESP32 hardware build pending; thermal and audio pending hardware.</t>
+          <t>MAIN .51 unavailable for centralized serial validation; NODE_02/NODE_03 ESP32 hardware not yet assembled.</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
@@ -9732,7 +9987,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>CSI camera .51/.52/.53/.54 PASS; remote aggregation PASS; serial hardware PASS; serial dashboard integration PENDING (blocked by .51 unavailability).</t>
+          <t>Firmware: 4-env build PASS. RPi: py_compile PASS. Tests: test_api_devices 7-logic PASS, test_lora_pipeline PASS. Pending: RPi live tests.</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -9800,7 +10055,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Verify MAIN ESP32 USB serial integration on .51 MAIN (blocked by .51 unavailability)</t>
+          <t>Wire ESP32 to NODE03 GPIO UART; verify NODE01/NODE02 UART readiness.</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
@@ -14447,6 +14702,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -14848,7 +15104,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Install USB microphone on a node and run detector.py with synthetic then field audio.</t>
+          <t>Device enumeration v2 fixed (non-zero arecord -l authoritative). Detector UX, sample rate, visualizer implemented. Pending: install USB mic on a node and run live field validation.</t>
         </is>
       </c>
     </row>
@@ -15935,7 +16191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.70000076293945" customWidth="1" min="1" max="1"/>
@@ -17826,6 +18082,258 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>C029</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Separate NODE dashboard for .52/.53/.54; MAIN preserved; simulation forced to live</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>node_dashboard.html; node_app.js; app.py; config.json</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>py_compile PASS</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>NODE GUI cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>C030</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Chainsaw detector UX: device selection, error visibility, Starting feedback, audio visualizer</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>detector.py; app.py; node_app.js</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>py_compile PASS</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Field validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>C031</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Sample rate fix: detector uses device default_samplerate (44100 Hz)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>detector.py</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Detector starts without PaError</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>a1907e3</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Test with other USB mic models</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>C032</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Live device enumeration: /api/devices uses arecord -l for ALSA query</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>app.py</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Empty arecord -&gt; empty device list</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2ab870f</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Field validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>C033</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Live device enumeration v2: non-zero arecord exit authoritative; regression tests</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>app.py; tests/test_api_devices.py</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>7 logic tests PASS</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>423fb63</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>RPi live validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>C034</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Firmware</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Multi-node firmware: 4 PlatformIO envs (main/node_01/node_02/node_03)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>main.cpp; platformio.ini</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>All 4 envs SUCCESS</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>daf78c4</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Flash when ESP32 arrives</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17837,7 +18345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -18210,6 +18718,141 @@
       <c r="E17" s="18" t="inlineStr">
         <is>
           <t>LoRa RX two-way MAIN ↔ NODE_01 validated (RSSI -29 to -35 dBm; SNR 9.25-10.00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Live device enumeration v2</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>arecord -l non-zero exit now authoritative; no stale PortAudio. tests/test_api_devices.py added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Firmware</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Multi-node firmware builds</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>4 PlatformIO envs produce distinct firmware.bin. Flash: 21.5%, RAM: 6.6%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>NODE03 UART readiness</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>/dev/serial0 exists; serial reader connected; local_serial.connected=true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>NODE_02/NODE_03 ESP32</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Firmware ready. ESP32 + LoRa + sensor modules not yet assembled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MAIN .51 availability</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>.51 unavailable. Centralized serial validation and multi-node integration blocked.</t>
         </is>
       </c>
     </row>

</xml_diff>